<commit_message>
Add partner api tests, add qa external to run tests against localhost
</commit_message>
<xml_diff>
--- a/defects/defects.xlsx
+++ b/defects/defects.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$O$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1426,8 +1426,1027 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>L37-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Orders in the same poll window as a partner API 500 are lost</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Partner API polling</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>When one poll of the partner API gets a 500, every order that happened upstream in that poll's time window is never picked up. The next poll starts after the failed window instead of retrying it. The orders are never stored and never made, and nothing is logged about them.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Partner API: "The API sometimes fails with a 500, and a retry of the same request succeeds. Nothing that happens upstream may be lost."
+- README, Mock partner API: "An enqueued response with a non-200 response is a transient upstream failure. The first poll whose window covers it gets that failure back. Retrying the same time_since succeeds and returns everything else enqueued in that window."</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Environment:
+- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
+- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
+- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
+Before you start:
+- OrderHub is stopped (Ctrl-C in the make run terminal).
+- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
+- No other traffic is sent to OrderHub or the mock while reproducing.
+Steps:
+1. Enqueue a 500 and an order on the mock, one right after the other (within 2 seconds, so both land in the same poll window). Run both lines together:
+curl -s -X POST localhost:8090/enqueue -d '{"response":500,"error":"Internal server error"}'
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-5005-1":{"order":5005,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"}}}'
+2. Confirm the mock recorded both: curl -s localhost:8090/status
+3. Wait 10 seconds (5 poll cycles).
+4. List partner orders: curl -s 'localhost:8080/api/orders?source=api' | python3 -m json.tool
+5. Control: enqueue a second order on its own, wait 4 seconds, and list again:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-5006-1":{"order":5006,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"}}}'
+curl -s 'localhost:8080/api/orders?source=api' | python3 -m json.tool
+6. Look at the OrderHub log in the make run terminal.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Failure response:
+{"response": 500, "error": "Internal server error"}
+Partner order 5005, sent in the same poll window:
+{
+  "response": 200,
+  "data": {
+    "i-5005-1": {"order": 5005, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"}
+  }
+}
+Control order 5006, sent later on its own:
+{
+  "response": 200,
+  "data": {
+    "i-5006-1": {"order": 5006, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"}
+  }
+}</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2: {"enqueued":2,"failures":1}.
+- The poll that gets the 500 is retried with the same time_since, as the spec describes. Order 5005 is picked up on the retry.
+- Step 4 lists order 5005.
+- Step 5 lists both 5005 and 5006.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2: {"enqueued":2,"failures":1}. The mock received both, so the order was available upstream.
+- The OrderHub log shows "poller: upstream returned 500: Internal server error", and there is no retry.
+- Step 4: no partner orders at all. Order 5005 is lost.
+- Step 5: only order 5006 appears. Polling itself recovered; only the failed window was skipped. 5005 never appears, even after waiting.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Mock responses and GET localhost:8090/status (steps 1 and 2):
+enqueued at 2026-09-27T21:55:10.524409898Z
+enqueued at 2026-09-27T21:55:10.531793697Z
+{"enqueued":2,"failures":1}
+GET /api/orders?source=api after 10 seconds (step 4):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": []
+}
+Control order 5006 enqueued on its own (step 5):
+enqueued at 2026-09-27T21:55:20.588867144Z
+GET /api/orders?source=api (step 5):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 1,
+            "source": "api",
+            "external_id": "5006",
+            "platform": "Partner API",
+            "restaurant": "",
+            "customer_first": "",
+            "customer_last": "",
+            "items": [
+                {
+                    "key": "i-5006-1",
+                    "name": "Cold brew",
+                    "category": "Coffee &amp; Tea",
+                    "price": 4.25,
+                    "status": "ordered"
+                }
+            ],
+            "notes": "",
+            "total": 4.25,
+            "status": "dispatched",
+            "ready_at": "2026-09-27 21:55:20",
+            "created_at": "2026-09-27 21:55:20",
+            "updated_at": "2026-09-27 21:55:22"
+        }
+    ]
+}
+OrderHub log:
+2026/09/27 14:55:08 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 14:55:08 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 14:55:08 poller: polling http://localhost:8090 every 2s
+2026/09/27 14:55:10 poller: upstream returned 500: Internal server error
+2026/09/27 14:55:22 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>- Every order that happened upstream while a poll failed is silently lost: never stored, never made, no alert. The spec says 500s happen "sometimes", so this will happen in production.
+- The more orders arrive per 2-second window (bursts), the more are lost per failure.
+- Status updates and cancellations in that window are lost too, so a cancelled order may still be made.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>- Black-box inference: after a failed poll, the next poll seems to ask for changes since the time of the failed poll, not since the last successful one. The mock is built to succeed when the same time_since is retried, so a retry would recover everything.
+- Related: restarting OrderHub may lose orders the same way (what happened upstream while it was down). To be tested in the restart tests.</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_partner_api.py -k same_window_as_a_500 must pass (remove the xfail marker once it reports XPASS(strict)).
+- tests/test_partner_api.py::test_polling_recovers_after_a_500 must still pass.</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_partner_api.py::test_order_in_the_same_window_as_a_500_is_not_lost</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>L37-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>A partner API update for some of an order's items removes the other items</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Partner API merging</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>The partner API only sends the items that changed. When an update arrives for one item of a two-item order, OrderHub replaces the order's item list with just that one item. The other item disappears from the order and the total drops to the price of the updated item.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Partner API: "The response contains every item that changed since time_since ... A response only contains the items that changed."
+- README, Payload formats, Partner API: "Each key in data is an item id. Items belong to orders via order."</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Environment:
+- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
+- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
+- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
+Before you start:
+- OrderHub is stopped (Ctrl-C in the make run terminal).
+- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
+- No other traffic is sent to OrderHub or the mock while reproducing.
+Steps:
+1. Enqueue partner order 6006 with two items:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-6006-1":{"order":6006,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"},"i-6006-2":{"order":6006,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"ordered"}}}'
+2. Wait 4 seconds, then show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+3. Enqueue a status update for Cold brew only (processing):
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-6006-1":{"order":6006,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"processing"}}}'
+4. Wait 4 seconds, then show the order again: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+5. Show its history: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+6. Show what the robot received: cat data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Order 6006, first response:
+{
+  "response": 200,
+  "data": {
+    "i-6006-1": {"order": 6006, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"},
+    "i-6006-2": {"order": 6006, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "ordered"}
+  }
+}
+Update for one item:
+{
+  "response": 200,
+  "data": {
+    "i-6006-1": {"order": 6006, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "processing"}
+  }
+}</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2: order 6006 with Blueberry pancakes and Cold brew, total 15.75.
+- Step 4: still both items, Cold brew now processing, Blueberry pancakes still ordered, total 15.75.
+- Step 5: an upstream_update event for Cold brew.</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2: correct, both items, total 15.75, dispatched.
+- Step 4: only Cold brew (processing). Blueberry pancakes is gone from the order and the total is 4.25.
+- Step 5: the upstream_update event only mentions Cold brew; there is no event saying Blueberry pancakes was removed.
+- Step 6: the robot did get both items, because the order was dispatched before the update arrived.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/orders/1 before the update (step 2):
+{
+    "id": 1,
+    "source": "api",
+    "external_id": "6006",
+    "platform": "Partner API",
+    "restaurant": "",
+    "customer_first": "",
+    "customer_last": "",
+    "items": [
+        {
+            "key": "i-6006-2",
+            "name": "Blueberry pancakes",
+            "category": "Breakfast",
+            "price": 11.5,
+            "status": "ordered"
+        },
+        {
+            "key": "i-6006-1",
+            "name": "Cold brew",
+            "category": "Coffee &amp; Tea",
+            "price": 4.25,
+            "status": "ordered"
+        }
+    ],
+    "notes": "",
+    "total": 15.75,
+    "status": "dispatched",
+    "ready_at": "2026-09-27 21:55:27",
+    "created_at": "2026-09-27 21:55:27",
+    "updated_at": "2026-09-27 21:55:28"
+}
+enqueued at 2026-09-27T21:55:30.723173904Z
+GET /api/orders/1 after the update (step 4):
+{
+    "id": 1,
+    "source": "api",
+    "external_id": "6006",
+    "platform": "Partner API",
+    "restaurant": "",
+    "customer_first": "",
+    "customer_last": "",
+    "items": [
+        {
+            "key": "i-6006-1",
+            "name": "Cold brew",
+            "category": "Coffee &amp; Tea",
+            "price": 4.25,
+            "status": "processing"
+        }
+    ],
+    "notes": "",
+    "total": 4.25,
+    "status": "dispatched",
+    "ready_at": "2026-09-27 21:55:27",
+    "created_at": "2026-09-27 21:55:27",
+    "updated_at": "2026-09-27 21:55:31"
+}
+GET /api/orders/1/events (step 5):
+{
+    "events": [
+        {
+            "id": 1,
+            "order_id": 1,
+            "kind": "received",
+            "detail": {
+                "items": [
+                    {
+                        "key": "i-6006-2",
+                        "name": "Blueberry pancakes",
+                        "category": "Breakfast",
+                        "price": 11.5,
+                        "status": "ordered"
+                    },
+                    {
+                        "key": "i-6006-1",
+                        "name": "Cold brew",
+                        "category": "Coffee &amp; Tea",
+                        "price": 4.25,
+                        "status": "ordered"
+                    }
+                ],
+                "order": 6006
+            },
+            "created_at": "2026-09-27 21:55:27"
+        },
+        {
+            "id": 2,
+            "order_id": 1,
+            "kind": "dispatched",
+            "detail": {
+                "dispatch_id": "ab4ecf0d4cc3b632",
+                "order_id": 1,
+                "external_ref": "api:6006",
+                "source": "api",
+                "station": "assembly-1",
+                "customer": " ",
+                "items": [
+                    {
+                        "line": 1,
+                        "name": "Blueberry pancakes",
+                        "qty": 1
+                    },
+                    {
+                        "line": 2,
+                        "name": "Cold brew",
+                        "qty": 1
+                    }
+                ],
+                "dispatch_at": "2026-09-27T21:55:28Z"
+            },
+            "created_at": "2026-09-27 21:55:28"
+        },
+        {
+            "id": 3,
+            "order_id": 1,
+            "kind": "upstream_update",
+            "detail": {
+                "statuses": {
+                    "Cold brew": "processing"
+                }
+            },
+            "created_at": "2026-09-27 21:55:31"
+        }
+    ]
+}
+data/robot_dispatch.jsonl (step 6):
+{"dispatch_id":"ab4ecf0d4cc3b632","order_id":1,"external_ref":"api:6006","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-27T21:55:28Z"}
+OrderHub log:
+2026/09/27 14:55:25 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 14:55:25 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 14:55:25 poller: polling http://localhost:8090 every 2s
+2026/09/27 14:55:28 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>- The stored order no longer matches what the customer ordered or what the robot made. Operators, support and any reporting built on totals see the wrong items and the wrong amount.
+- Every normal status update (processing, with_courier, delivered) usually touches only some items, so this happens on almost every multi-item partner order.
+- It causes L37-007: after an update for one cancelled item, the order only "has" cancelled items and is treated as fully cancelled.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>- If an update arrives before the order is dispatched, the robot would receive only the updated items. With a 1-second dispatcher that window is small, but it grows when the dispatcher is slow or backed up.
+- Related: L37-007 (same cause), L37-009.</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_partner_api.py -k keeps_the_other_items must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_partner_api.py::test_status_update_for_one_item_keeps_the_other_items</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>L37-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Cancelling one item of a partner order cancels the whole order, even after it was made</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Partner API merging, cancellation</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>When the partner API cancels one item of a two-item order, OrderHub cancels the whole order. The order had already been sent to the robot, so it now shows as cancelled although the food was made.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>- README, Payload formats, Partner API: "An order whose items are all cancelled is cancelled." So an order with some items cancelled is not cancelled.
+- README, Order lifecycle: "Once an order is dispatched, the robot is already building it, so it can no longer be cancelled."</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Environment:
+- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
+- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
+- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
+Before you start:
+- OrderHub is stopped (Ctrl-C in the make run terminal).
+- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
+- No other traffic is sent to OrderHub or the mock while reproducing.
+Steps:
+1. Enqueue partner order 7007 with two items:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-7007-1":{"order":7007,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"},"i-7007-2":{"order":7007,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"ordered"}}}'
+2. Wait 4 seconds, then show the order (it is dispatched): curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+3. Enqueue a cancel for Blueberry pancakes only:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-7007-2":{"order":7007,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"cancelled"}}}'
+4. Wait 4 seconds, then show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+5. Show its history: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+6. Show what the robot received: cat data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Order 7007, first response:
+{
+  "response": 200,
+  "data": {
+    "i-7007-1": {"order": 7007, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"},
+    "i-7007-2": {"order": 7007, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "ordered"}
+  }
+}
+Cancel for one item:
+{
+  "response": 200,
+  "data": {
+    "i-7007-2": {"order": 7007, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "cancelled"}
+  }
+}</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>- Step 4: the order is still dispatched. Cold brew is still ordered; Blueberry pancakes is cancelled.
+- Step 5: an upstream_update event for Blueberry pancakes, and no cancelled event for the order.
+- Because the order was already dispatched, it must not become cancelled even if all items were cancelled.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2: dispatched, both items, total 15.75.
+- Step 4: status cancelled. Only Blueberry pancakes (cancelled) is left on the order; Cold brew is gone. Total 11.5.
+- Step 5: upstream_update for Blueberry pancakes, then cancelled by partner-api.
+- Step 6: the robot had already received both items. The order shows cancelled although it was made.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/orders/1 before the cancel (step 2):
+{
+    "id": 1,
+    "source": "api",
+    "external_id": "7007",
+    "platform": "Partner API",
+    "restaurant": "",
+    "customer_first": "",
+    "customer_last": "",
+    "items": [
+        {
+            "key": "i-7007-2",
+            "name": "Blueberry pancakes",
+            "category": "Breakfast",
+            "price": 11.5,
+            "status": "ordered"
+        },
+        {
+            "key": "i-7007-1",
+            "name": "Cold brew",
+            "category": "Coffee &amp; Tea",
+            "price": 4.25,
+            "status": "ordered"
+        }
+    ],
+    "notes": "",
+    "total": 15.75,
+    "status": "dispatched",
+    "ready_at": "2026-09-27 21:55:37",
+    "created_at": "2026-09-27 21:55:37",
+    "updated_at": "2026-09-27 21:55:38"
+}
+enqueued at 2026-09-27T21:55:40.900354587Z
+GET /api/orders/1 after the cancel (step 4):
+{
+    "id": 1,
+    "source": "api",
+    "external_id": "7007",
+    "platform": "Partner API",
+    "restaurant": "",
+    "customer_first": "",
+    "customer_last": "",
+    "items": [
+        {
+            "key": "i-7007-2",
+            "name": "Blueberry pancakes",
+            "category": "Breakfast",
+            "price": 11.5,
+            "status": "cancelled"
+        }
+    ],
+    "notes": "",
+    "total": 11.5,
+    "status": "cancelled",
+    "ready_at": "2026-09-27 21:55:37",
+    "created_at": "2026-09-27 21:55:37",
+    "updated_at": "2026-09-27 21:55:41"
+}
+GET /api/orders/1/events (step 5):
+{
+    "events": [
+        {
+            "id": 1,
+            "order_id": 1,
+            "kind": "received",
+            "detail": {
+                "items": [
+                    {
+                        "key": "i-7007-2",
+                        "name": "Blueberry pancakes",
+                        "category": "Breakfast",
+                        "price": 11.5,
+                        "status": "ordered"
+                    },
+                    {
+                        "key": "i-7007-1",
+                        "name": "Cold brew",
+                        "category": "Coffee &amp; Tea",
+                        "price": 4.25,
+                        "status": "ordered"
+                    }
+                ],
+                "order": 7007
+            },
+            "created_at": "2026-09-27 21:55:37"
+        },
+        {
+            "id": 2,
+            "order_id": 1,
+            "kind": "dispatched",
+            "detail": {
+                "dispatch_id": "7cc3b56bcb111c81",
+                "order_id": 1,
+                "external_ref": "api:7007",
+                "source": "api",
+                "station": "assembly-1",
+                "customer": " ",
+                "items": [
+                    {
+                        "line": 1,
+                        "name": "Blueberry pancakes",
+                        "qty": 1
+                    },
+                    {
+                        "line": 2,
+                        "name": "Cold brew",
+                        "qty": 1
+                    }
+                ],
+                "dispatch_at": "2026-09-27T21:55:38Z"
+            },
+            "created_at": "2026-09-27 21:55:38"
+        },
+        {
+            "id": 3,
+            "order_id": 1,
+            "kind": "upstream_update",
+            "detail": {
+                "statuses": {
+                    "Blueberry pancakes": "cancelled"
+                }
+            },
+            "created_at": "2026-09-27 21:55:41"
+        },
+        {
+            "id": 4,
+            "order_id": 1,
+            "kind": "cancelled",
+            "detail": {
+                "by": "partner-api"
+            },
+            "created_at": "2026-09-27 21:55:41"
+        }
+    ]
+}
+data/robot_dispatch.jsonl (step 6):
+{"dispatch_id":"7cc3b56bcb111c81","order_id":1,"external_ref":"api:7007","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-27T21:55:38Z"}
+OrderHub log:
+2026/09/27 14:55:35 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 14:55:35 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 14:55:35 poller: polling http://localhost:8090 every 2s
+2026/09/27 14:55:38 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>- A customer who removed one item has their whole order marked cancelled. Support and the platform would treat it as not delivered or refund it, while the food was made.
+- The order history says the partner cancelled the order, which is not what happened.
+- It also shows a dispatched order being moved to cancelled, which the spec forbids.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>- Black-box inference: this is a result of L37-006. After the update, the order only contains the cancelled item, so "all items cancelled" is true. Fixing L37-006 likely fixes the first part.
+- The second part (a dispatched order can still become cancelled) is separate and also happens through the operator cancel API. To be covered in the dispatch tests.
+- Related: L37-006.</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_partner_api.py -k cancelling_one_item must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_partner_api.py::test_cancelling_one_item_does_not_cancel_the_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>L37-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>A partner order that arrives with every item cancelled is made</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Partner API merging, cancellation</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>If OrderHub first sees a partner order when all its items are already cancelled (the customer cancelled before the next poll), it creates the order as queued and sends it to the robot. The cancelled status of the items is ignored.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>- README, Payload formats, Partner API: "An order whose items are all cancelled is cancelled."
+- README, Order lifecycle: "A cancelled order is never dispatched."
+- The poll interval is 2 seconds and the mock merges everything in a window into one response, so an order and its cancellation can arrive in the same poll.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Environment:
+- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
+- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
+- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
+Before you start:
+- OrderHub is stopped (Ctrl-C in the make run terminal).
+- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
+- No other traffic is sent to OrderHub or the mock while reproducing.
+Steps:
+1. Enqueue partner order 8008 with both items already cancelled:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-8008-1":{"order":8008,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"cancelled"},"i-8008-2":{"order":8008,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"cancelled"}}}'
+2. Wait 5 seconds.
+3. Show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+4. Show its history: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+5. Show what the robot received: cat data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "response": 200,
+  "data": {
+    "i-8008-1": {"order": 8008, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "cancelled"},
+    "i-8008-2": {"order": 8008, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "cancelled"}
+  }
+}</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>- The order is created as cancelled (or not created at all).
+- It is never sent to the robot. data/robot_dispatch.jsonl is empty.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>- Step 3: the order is dispatched. Both items show status cancelled, and the total is 15.75.
+- Step 4: received, then dispatched. No cancelled event.
+- Step 5: the robot received Blueberry pancakes and Cold brew.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/orders/1 (step 3):
+{
+    "id": 1,
+    "source": "api",
+    "external_id": "8008",
+    "platform": "Partner API",
+    "restaurant": "",
+    "customer_first": "",
+    "customer_last": "",
+    "items": [
+        {
+            "key": "i-8008-2",
+            "name": "Blueberry pancakes",
+            "category": "Breakfast",
+            "price": 11.5,
+            "status": "cancelled"
+        },
+        {
+            "key": "i-8008-1",
+            "name": "Cold brew",
+            "category": "Coffee &amp; Tea",
+            "price": 4.25,
+            "status": "cancelled"
+        }
+    ],
+    "notes": "",
+    "total": 15.75,
+    "status": "dispatched",
+    "ready_at": "2026-09-27 21:55:47",
+    "created_at": "2026-09-27 21:55:47",
+    "updated_at": "2026-09-27 21:55:48"
+}
+GET /api/orders/1/events (step 4):
+{
+    "events": [
+        {
+            "id": 1,
+            "order_id": 1,
+            "kind": "received",
+            "detail": {
+                "items": [
+                    {
+                        "key": "i-8008-2",
+                        "name": "Blueberry pancakes",
+                        "category": "Breakfast",
+                        "price": 11.5,
+                        "status": "cancelled"
+                    },
+                    {
+                        "key": "i-8008-1",
+                        "name": "Cold brew",
+                        "category": "Coffee &amp; Tea",
+                        "price": 4.25,
+                        "status": "cancelled"
+                    }
+                ],
+                "order": 8008
+            },
+            "created_at": "2026-09-27 21:55:47"
+        },
+        {
+            "id": 2,
+            "order_id": 1,
+            "kind": "dispatched",
+            "detail": {
+                "dispatch_id": "69ca66b7ed464e31",
+                "order_id": 1,
+                "external_ref": "api:8008",
+                "source": "api",
+                "station": "assembly-1",
+                "customer": " ",
+                "items": [
+                    {
+                        "line": 1,
+                        "name": "Blueberry pancakes",
+                        "qty": 1
+                    },
+                    {
+                        "line": 2,
+                        "name": "Cold brew",
+                        "qty": 1
+                    }
+                ],
+                "dispatch_at": "2026-09-27T21:55:48Z"
+            },
+            "created_at": "2026-09-27 21:55:48"
+        }
+    ]
+}
+data/robot_dispatch.jsonl (step 5):
+{"dispatch_id":"69ca66b7ed464e31","order_id":1,"external_ref":"api:8008","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-27T21:55:48Z"}
+OrderHub log:
+2026/09/27 14:55:45 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 14:55:45 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 14:55:45 poller: polling http://localhost:8090 every 2s
+2026/09/27 14:55:48 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>- A fully cancelled order is made. Food and robot time are wasted.
+- The same happens whenever an order and its cancellation fall into the same 2-second poll window, or when OrderHub first sees the order after a failed poll (L37-005).</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>- Black-box inference: the "all items cancelled" rule seems to be applied only to orders OrderHub already knows, not to orders it sees for the first time.
+- The total includes the cancelled items (see also L37-009).
+- Related: L37-005, L37-009.</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_partner_api.py -k fully_cancelled must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_partner_api.py::test_order_that_arrives_fully_cancelled_is_never_dispatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>L37-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Cancelled items of a partner order are sent to the robot</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Partner API merging, robot payload</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>A partner order with one ordered item and one cancelled item is sent to the robot with both items. The robot makes the cancelled item.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>- README, Payload formats, Partner API: item status "moves through ordered, processing, with_courier, and delivered, or becomes cancelled".
+- README, Order lifecycle: "A cancelled order is never dispatched." The spec does not spell out item-level cancellation, but making an item the customer cancelled contradicts the intent. Question for the team to confirm.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Environment:
+- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
+- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
+- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
+Before you start:
+- OrderHub is stopped (Ctrl-C in the make run terminal).
+- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
+- No other traffic is sent to OrderHub or the mock while reproducing.
+Steps:
+1. Enqueue partner order 9009 with Cold brew ordered and Blueberry pancakes cancelled:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-9009-1":{"order":9009,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"},"i-9009-2":{"order":9009,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"cancelled"}}}'
+2. Wait 5 seconds.
+3. Show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+4. Show what the robot received: cat data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>{
+  "response": 200,
+  "data": {
+    "i-9009-1": {"order": 9009, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"},
+    "i-9009-2": {"order": 9009, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "cancelled"}
+  }
+}</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>- The robot receives only Cold brew.
+- The order total is 4.25 (cancelled items not counted), or the team confirms how totals should treat cancelled items.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>- Step 3: the order is dispatched with both items; Blueberry pancakes shows cancelled. Total 15.75.
+- Step 4: the robot received Blueberry pancakes and Cold brew. The robot payload has no item status, so the robot cannot tell the pancakes were cancelled.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/orders/1 (step 3):
+{
+    "id": 1,
+    "source": "api",
+    "external_id": "9009",
+    "platform": "Partner API",
+    "restaurant": "",
+    "customer_first": "",
+    "customer_last": "",
+    "items": [
+        {
+            "key": "i-9009-2",
+            "name": "Blueberry pancakes",
+            "category": "Breakfast",
+            "price": 11.5,
+            "status": "cancelled"
+        },
+        {
+            "key": "i-9009-1",
+            "name": "Cold brew",
+            "category": "Coffee &amp; Tea",
+            "price": 4.25,
+            "status": "ordered"
+        }
+    ],
+    "notes": "",
+    "total": 15.75,
+    "status": "dispatched",
+    "ready_at": "2026-09-27 21:55:54",
+    "created_at": "2026-09-27 21:55:54",
+    "updated_at": "2026-09-27 21:55:55"
+}
+data/robot_dispatch.jsonl (step 4):
+{"dispatch_id":"947dff8a958d0725","order_id":1,"external_ref":"api:9009","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-27T21:55:55Z"}
+OrderHub log:
+2026/09/27 14:55:52 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 14:55:52 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 14:55:52 poller: polling http://localhost:8090 every 2s
+2026/09/27 14:55:55 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>- The robot makes items the customer cancelled. Food and robot time are wasted, and the customer may be charged or refunded inconsistently.
+- The robot payload carries no item status, so nothing downstream can catch it.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>- Spec gap: item-level cancellation is not described explicitly. Worth confirming with the team; I treated it as a defect because a cancelled item should not be made.
+- Related: L37-006, L37-008.</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_partner_api.py -k cancelled_item_is_not_sent must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_partner_api.py::test_cancelled_item_is_not_sent_to_the_robot</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O5"/>
+  <autoFilter ref="A1:O10"/>
   <conditionalFormatting sqref="C2:C1000">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$C2="Critical"</formula>

</xml_diff>

<commit_message>
Add dispatch tests with slow and failing robots, 3 more bugs 010-012
</commit_message>
<xml_diff>
--- a/defects/defects.xlsx
+++ b/defects/defects.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$O$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,24 +465,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="90" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="90" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="90" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
     <col width="55" customWidth="1" min="13" max="13"/>
     <col width="55" customWidth="1" min="14" max="14"/>
-    <col width="45" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -498,34 +497,34 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Automated test</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Spec reference</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Steps to reproduce</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Test data</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Expected result</t>
@@ -554,11 +553,6 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>How to verify the fix</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Automated test</t>
         </is>
       </c>
     </row>
@@ -575,74 +569,47 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>tests/test_webhook.py::test_same_order_id_on_two_platforms_creates_two_orders</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Webhook ingest</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>When two delivery platforms send orders that happen to use the same order_id, OrderHub keeps only the first one. The second request is answered with 202 and the first order's id, its payload is written into the first order's history, and it is never stored as its own order or sent to the robot. The platform is told it succeeded, so it never retries.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>- README, How it's supposed to work, Pipelines, Webhook: "Each platform assigns its own order_ids."
 - README, Payload formats, Webhook: order_id is "Assigned by the platform"; order_source is "The platform: Grubstub, DoorDrop, or Overeats".
 So Grubstub order 1001 and DoorDrop order 1001 are two different orders from two different customers.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl).
-- Also reproduced by the automated test, which starts its own OrderHub on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run.
-- No other traffic is sent to OrderHub while reproducing.
-Steps:
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
 1. Send the Grubstub order:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' \
-  -d '{"order_id":"1001","order_source":"Grubstub","restaurant":"Just Pizza","first_name":"Gina","last_name":"Park","total":24.5,"items":["Margherita pizza"],"notes":""}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"1001","order_source":"Grubstub","restaurant":"Just Pizza","first_name":"Gina","last_name":"Park","total":24.5,"items":["Margherita pizza"],"notes":""}'
 2. Send the DoorDrop order with the same order_id:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' \
-  -d '{"order_id":"1001","order_source":"DoorDrop","restaurant":"Cluck Norris","first_name":"Dora","last_name":"Ortiz","total":18.75,"items":["Chicken sandwich"],"notes":""}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"1001","order_source":"DoorDrop","restaurant":"Cluck Norris","first_name":"Dora","last_name":"Ortiz","total":18.75,"items":["Chicken sandwich"],"notes":""}'
 3. Wait 3 seconds so the dispatcher can run.
-4. List webhook orders: curl -s 'localhost:8080/api/orders?source=webhook' | python3 -m json.tool
-5. Show the history of order 1: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
-6. Show the dashboard counts: curl -s localhost:8080/api/stats | python3 -m json.tool
-7. Show what the robot received: cat data/robot_dispatch.jsonl</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Grubstub order 1001, customer Gina Park:
-{
-  "order_id": "1001",
-  "order_source": "Grubstub",
-  "restaurant": "Just Pizza",
-  "first_name": "Gina",
-  "last_name": "Park",
-  "total": 24.5,
-  "items": ["Margherita pizza"],
-  "notes": ""
-}
-DoorDrop order 1001, customer Dora Ortiz:
-{
-  "order_id": "1001",
-  "order_source": "DoorDrop",
-  "restaurant": "Cluck Norris",
-  "first_name": "Dora",
-  "last_name": "Ortiz",
-  "total": 18.75,
-  "items": ["Chicken sandwich"],
-  "notes": ""
-}</t>
+4. List webhook orders:
+curl -s 'localhost:8080/api/orders?source=webhook' | python3 -m json.tool
+5. Show the history of order 1:
+curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+6. Show the dashboard counts:
+curl -s localhost:8080/api/stats | python3 -m json.tool
+7. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -664,10 +631,19 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>HTTP responses (steps 1 and 2):
-{"id":1} HTTP 202
-{"id":1} HTTP 202
-GET /api/orders?source=webhook (step 4):
+          <t>Step 1 (Send the Grubstub order):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:54:40 GMT
+Content-Length: 9
+{"id":1}
+Step 2 (Send the DoorDrop order with the same order_id):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:54:40 GMT
+Content-Length: 9
+{"id":1}
+Step 4 (List webhook orders):
 {
     "limit": 50,
     "offset": 0,
@@ -688,13 +664,13 @@
             "notes": "",
             "total": 24.5,
             "status": "dispatched",
-            "ready_at": "2026-09-27 20:27:54",
-            "created_at": "2026-09-27 20:27:54",
-            "updated_at": "2026-09-27 20:27:54"
+            "ready_at": "2026-09-28 03:54:40",
+            "created_at": "2026-09-28 03:54:40",
+            "updated_at": "2026-09-28 03:54:40"
         }
     ]
 }
-GET /api/orders/1/events (step 5):
+Step 5 (Show the history of order 1):
 {
     "events": [
         {
@@ -713,7 +689,7 @@
                 ],
                 "notes": ""
             },
-            "created_at": "2026-09-27 20:27:54"
+            "created_at": "2026-09-28 03:54:40"
         },
         {
             "id": 2,
@@ -731,14 +707,14 @@
                 ],
                 "notes": ""
             },
-            "created_at": "2026-09-27 20:27:54"
+            "created_at": "2026-09-28 03:54:40"
         },
         {
             "id": 3,
             "order_id": 1,
             "kind": "dispatched",
             "detail": {
-                "dispatch_id": "55bc0ed2b990b47a",
+                "dispatch_id": "007cf0a45e80156f",
                 "order_id": 1,
                 "external_ref": "webhook:1001",
                 "source": "webhook",
@@ -751,13 +727,13 @@
                         "qty": 1
                     }
                 ],
-                "dispatch_at": "2026-09-27T20:27:54Z"
+                "dispatch_at": "2026-09-28T03:54:40Z"
             },
-            "created_at": "2026-09-27 20:27:54"
+            "created_at": "2026-09-28 03:54:40"
         }
     ]
 }
-GET /api/stats (step 6):
+Step 6 (Show the dashboard counts):
 {
     "by_status": {
         "dispatched": 1
@@ -771,17 +747,17 @@
     "total_orders": 1,
     "total_events": 3,
     "last_hour": 1,
-    "refreshed_at": "2026-09-27T20:27:54Z"
+    "refreshed_at": "2026-09-28T03:54:40Z"
 }
-data/robot_dispatch.jsonl (step 7):
-{"dispatch_id":"55bc0ed2b990b47a","order_id":1,"external_ref":"webhook:1001","source":"webhook","station":"assembly-1","customer":"Gina Park","items":[{"line":1,"name":"Margherita pizza","qty":1}],"dispatch_at":"2026-09-27T20:27:54Z"}
-OrderHub log:
-2026/09/27 13:27:52 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 13:27:52 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 13:27:52 poller: polling http://localhost:8090 every 2s
-2026/09/27 13:27:54 POST /webhooks/orders 1ms
-2026/09/27 13:27:54 POST /webhooks/orders 0s
-2026/09/27 13:27:54 dispatch: sent 1 orders</t>
+Step 7 (Show what the robot received):
+{"dispatch_id":"007cf0a45e80156f","order_id":1,"external_ref":"webhook:1001","source":"webhook","station":"assembly-1","customer":"Gina Park","items":[{"line":1,"name":"Margherita pizza","qty":1}],"dispatch_at":"2026-09-28T03:54:40Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:54:38 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:54:38 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:54:38 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:54:40 POST /webhooks/orders 1ms
+2026/09/27 20:54:40 POST /webhooks/orders 0s
+2026/09/27 20:54:40 dispatch: sent 1 orders</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -805,11 +781,6 @@
 - Also check a retry of the same platform's order still creates one order: tests/test_webhook.py::test_retried_webhook_creates_one_order.</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_webhook.py::test_same_order_id_on_two_platforms_creates_two_orders</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="150" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -824,67 +795,44 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>tests/test_webhook.py::test_cancel_from_another_platform_does_not_cancel_the_order</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Webhook ingest, cancellation</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>A cancel message from DoorDrop for DoorDrop order 2002 cancels Grubstub's order 2002, which DoorDrop has nothing to do with. The cancel returns 202 with the Grubstub order's id, the history records it as cancelled by DoorDrop, and the order is never made.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>- README, How it's supposed to work, Pipelines, Webhook: 'A payload with "update": ["cancelled"] cancels an order that platform sent earlier. Each platform assigns its own order_ids.'</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl).
-- Also reproduced by the automated test, which starts its own OrderHub on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run.
-- No other traffic is sent to OrderHub while reproducing.
-Steps:
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
 1. Send the Grubstub order:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' \
-  -d '{"order_id":"2002","order_source":"Grubstub","restaurant":"Just Pizza","first_name":"Ada","last_name":"Park","total":24.5,"items":["Margherita pizza"],"notes":""}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"2002","order_source":"Grubstub","restaurant":"Just Pizza","first_name":"Ada","last_name":"Park","total":24.5,"items":["Margherita pizza"],"notes":""}'
 2. Immediately send the DoorDrop cancel:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' \
-  -d '{"order_id":"2002","order_source":"DoorDrop","update":["cancelled"]}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"2002","order_source":"DoorDrop","update":["cancelled"]}'
 3. Wait 3 seconds so the dispatcher can run.
-4. Show the Grubstub order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
-5. Show its history: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
-6. Show what the robot received: cat data/robot_dispatch.jsonl
+4. Show the Grubstub order:
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+5. Show its history:
+curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+6. Show what the robot received:
+cat data/robot_dispatch.jsonl
 Note: step 2 must happen within about a second of step 1, before the order is dispatched. If the order is already dispatched, the cancel still flips its status to cancelled (see Notes).</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Grubstub order 2002, customer Ada Park:
-{
-  "order_id": "2002",
-  "order_source": "Grubstub",
-  "restaurant": "Just Pizza",
-  "first_name": "Ada",
-  "last_name": "Park",
-  "total": 24.5,
-  "items": ["Margherita pizza"],
-  "notes": ""
-}
-DoorDrop cancel for DoorDrop order 2002 (OrderHub never received a DoorDrop order 2002):
-{
-  "order_id": "2002",
-  "order_source": "DoorDrop",
-  "update": ["cancelled"]
-}</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -905,10 +853,19 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>HTTP responses (steps 1 and 2):
-{"id":1} HTTP 202
-{"id":1} HTTP 202
-GET /api/orders/1 (step 4):
+          <t>Step 1 (Send the Grubstub order):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:54:46 GMT
+Content-Length: 9
+{"id":1}
+Step 2 (Immediately send the DoorDrop cancel):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:54:46 GMT
+Content-Length: 9
+{"id":1}
+Step 4 (Show the Grubstub order):
 {
     "id": 1,
     "source": "webhook",
@@ -925,11 +882,11 @@
     "notes": "",
     "total": 24.5,
     "status": "cancelled",
-    "ready_at": "2026-09-27 20:27:59",
-    "created_at": "2026-09-27 20:27:59",
-    "updated_at": "2026-09-27 20:27:59"
+    "ready_at": "2026-09-28 03:54:46",
+    "created_at": "2026-09-28 03:54:46",
+    "updated_at": "2026-09-28 03:54:46"
 }
-GET /api/orders/1/events (step 5):
+Step 5 (Show its history):
 {
     "events": [
         {
@@ -948,7 +905,7 @@
                 ],
                 "notes": ""
             },
-            "created_at": "2026-09-27 20:27:59"
+            "created_at": "2026-09-28 03:54:46"
         },
         {
             "id": 2,
@@ -957,18 +914,18 @@
             "detail": {
                 "by": "DoorDrop"
             },
-            "created_at": "2026-09-27 20:27:59"
+            "created_at": "2026-09-28 03:54:46"
         }
     ]
 }
-data/robot_dispatch.jsonl (step 6):
-(robot lines: 0)
-OrderHub log:
-2026/09/27 13:27:57 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 13:27:57 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 13:27:57 poller: polling http://localhost:8090 every 2s
-2026/09/27 13:27:59 POST /webhooks/orders 1ms
-2026/09/27 13:27:59 POST /webhooks/orders 0s</t>
+Step 6 (Show what the robot received):
+(empty: the robot received nothing)
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:54:44 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:54:44 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:54:44 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:54:46 POST /webhooks/orders 1ms
+2026/09/27 20:54:46 POST /webhooks/orders 1ms</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -992,11 +949,6 @@
 - Also check that a cancel from the same platform still works.</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_webhook.py::test_cancel_from_another_platform_does_not_cancel_the_order</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="150" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1011,68 +963,45 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>tests/test_webhook.py::test_cancel_that_arrives_first_still_cancels_the_order</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Webhook ingest, cancellation</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>If a platform's cancel reaches OrderHub before the order itself (possible because platforms retry failed requests), OrderHub answers the cancel with 202 and discards it. When the order arrives a moment later, it is created normally and sent to the robot. The cancel is not recorded anywhere.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>- README, How it's supposed to work, Order lifecycle: "A cancelled order is never dispatched."
 - README, Pipelines, Webhook: "Platforms retry on failure, so the same request may arrive more than once."
 Because platforms retry, requests can arrive out of order: the order request can fail and be retried after the customer has already cancelled.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl).
-- Also reproduced by the automated test, which starts its own OrderHub on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run.
-- No other traffic is sent to OrderHub while reproducing.
-Steps:
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
 1. Send the cancel:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' \
-  -d '{"order_id":"3003","order_source":"Overeats","update":["cancelled"]}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"3003","order_source":"Overeats","update":["cancelled"]}'
 2. Send the order:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' \
-  -d '{"order_id":"3003","order_source":"Overeats","restaurant":"Taco Place","first_name":"Lee","last_name":"Wong","total":12,"items":["Taco"],"notes":""}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"3003","order_source":"Overeats","restaurant":"Taco Place","first_name":"Lee","last_name":"Wong","total":12,"items":["Taco"],"notes":""}'
 3. Wait 3 seconds so the dispatcher can run.
-4. Show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
-5. Show its history: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
-6. Show what the robot received: cat data/robot_dispatch.jsonl</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Overeats cancel for order 3003, sent first:
-{
-  "order_id": "3003",
-  "order_source": "Overeats",
-  "update": ["cancelled"]
-}
-The Overeats order 3003 itself (the retry), sent second:
-{
-  "order_id": "3003",
-  "order_source": "Overeats",
-  "restaurant": "Taco Place",
-  "first_name": "Lee",
-  "last_name": "Wong",
-  "total": 12,
-  "items": ["Taco"],
-  "notes": ""
-}</t>
+4. Show the order:
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+5. Show its history:
+curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+6. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -1094,10 +1023,17 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>HTTP responses (steps 1 and 2):
-HTTP 202
-{"id":1} HTTP 202
-GET /api/orders/1 (step 4):
+          <t>Step 1 (Send the cancel):
+HTTP/1.1 202 Accepted
+Date: Mon, 28 Sep 2026 03:54:52 GMT
+Content-Length: 0
+Step 2 (Send the order):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:54:52 GMT
+Content-Length: 9
+{"id":1}
+Step 4 (Show the order):
 {
     "id": 1,
     "source": "webhook",
@@ -1114,11 +1050,11 @@
     "notes": "",
     "total": 12,
     "status": "dispatched",
-    "ready_at": "2026-09-27 20:28:04",
-    "created_at": "2026-09-27 20:28:04",
-    "updated_at": "2026-09-27 20:28:04"
+    "ready_at": "2026-09-28 03:54:52",
+    "created_at": "2026-09-28 03:54:52",
+    "updated_at": "2026-09-28 03:54:53"
 }
-GET /api/orders/1/events (step 5):
+Step 5 (Show its history):
 {
     "events": [
         {
@@ -1137,14 +1073,14 @@
                 ],
                 "notes": ""
             },
-            "created_at": "2026-09-27 20:28:04"
+            "created_at": "2026-09-28 03:54:52"
         },
         {
             "id": 2,
             "order_id": 1,
             "kind": "dispatched",
             "detail": {
-                "dispatch_id": "83fb4224a22d083c",
+                "dispatch_id": "69d8b5f90f6e2e9b",
                 "order_id": 1,
                 "external_ref": "webhook:3003",
                 "source": "webhook",
@@ -1157,22 +1093,22 @@
                         "qty": 1
                     }
                 ],
-                "dispatch_at": "2026-09-27T20:28:04Z"
+                "dispatch_at": "2026-09-28T03:54:53Z"
             },
-            "created_at": "2026-09-27 20:28:04"
+            "created_at": "2026-09-28 03:54:53"
         }
     ]
 }
-data/robot_dispatch.jsonl (step 6):
-{"dispatch_id":"83fb4224a22d083c","order_id":1,"external_ref":"webhook:3003","source":"webhook","station":"assembly-1","customer":"Lee Wong","items":[{"line":1,"name":"Taco","qty":1}],"dispatch_at":"2026-09-27T20:28:04Z"}
-OrderHub log:
-2026/09/27 13:28:02 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 13:28:02 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 13:28:02 poller: polling http://localhost:8090 every 2s
-2026/09/27 13:28:04 webhook: update for unknown order 3003
-2026/09/27 13:28:04 POST /webhooks/orders 0s
-2026/09/27 13:28:04 POST /webhooks/orders 0s
-2026/09/27 13:28:04 dispatch: sent 1 orders</t>
+Step 6 (Show what the robot received):
+{"dispatch_id":"69d8b5f90f6e2e9b","order_id":1,"external_ref":"webhook:3003","source":"webhook","station":"assembly-1","customer":"Lee Wong","items":[{"line":1,"name":"Taco","qty":1}],"dispatch_at":"2026-09-28T03:54:53Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:54:51 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:54:51 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:54:51 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:54:52 webhook: update for unknown order 3003
+2026/09/27 20:54:52 POST /webhooks/orders 0s
+2026/09/27 20:54:52 POST /webhooks/orders 0s
+2026/09/27 20:54:53 dispatch: sent 1 orders</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1195,11 +1131,6 @@
 - python -m pytest tests/test_webhook.py -k cancel_that_arrives_first must pass (remove the xfail marker once it reports XPASS(strict)).</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_webhook.py::test_cancel_that_arrives_first_still_cancels_the_order</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="150" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -1214,73 +1145,46 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>tests/test_webhook.py::test_webhook_with_missing_fields_is_rejected</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Webhook ingest, input validation</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>OrderHub accepts webhook requests with no order_id, no order_source and no items. An empty {} body creates a blank order that is sent to the robot with "items": null. Every later order without an order_id is answered with that blank order's id and merged into it, so real customer orders are silently lost.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>- README, Payload formats, Webhook: every order has order_id ("Assigned by the platform"), order_source ("Grubstub, DoorDrop, or Overeats"), and items ("One entry per item").
 - QA_HOMEWORK, Bad data: "OrderHub should be resilient to malformed and adversarial input."</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl).
-- Also reproduced by the automated test, which starts its own OrderHub on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run.
-- No other traffic is sent to OrderHub while reproducing.
-Steps:
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
 1. Send an empty JSON object:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{}'
 2. Send Ann's order without order_id:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' \
-  -d '{"order_source":"Grubstub","restaurant":"Soup Shack","first_name":"Ann","last_name":"Lee","total":8,"items":["Tomato soup"],"notes":""}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_source":"Grubstub","restaurant":"Soup Shack","first_name":"Ann","last_name":"Lee","total":8,"items":["Tomato soup"],"notes":""}'
 3. Send Bob's order without order_id:
-curl -s -w ' HTTP %{http_code}\n' -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' \
-  -d '{"order_source":"DoorDrop","restaurant":"Green Bowl","first_name":"Bob","last_name":"Diaz","total":11,"items":["Caesar salad"],"notes":""}'
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_source":"DoorDrop","restaurant":"Green Bowl","first_name":"Bob","last_name":"Diaz","total":11,"items":["Caesar salad"],"notes":""}'
 4. Wait 3 seconds so the dispatcher can run.
-5. List orders: curl -s localhost:8080/api/orders | python3 -m json.tool
-6. Show the history of order 1: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
-7. Show what the robot received: cat data/robot_dispatch.jsonl</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>1. An empty JSON object: {}
-2. Ann Lee's order from Grubstub, missing order_id:
-{
-  "order_source": "Grubstub",
-  "restaurant": "Soup Shack",
-  "first_name": "Ann",
-  "last_name": "Lee",
-  "total": 8,
-  "items": ["Tomato soup"],
-  "notes": ""
-}
-3. Bob Diaz's order from DoorDrop, missing order_id:
-{
-  "order_source": "DoorDrop",
-  "restaurant": "Green Bowl",
-  "first_name": "Bob",
-  "last_name": "Diaz",
-  "total": 11,
-  "items": ["Caesar salad"],
-  "notes": ""
-}</t>
+5. List orders:
+curl -s localhost:8080/api/orders | python3 -m json.tool
+6. Show the history of order 1:
+curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+7. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1299,11 +1203,25 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>HTTP responses (steps 1 to 3):
-{"id":1} HTTP 202
-{"id":1} HTTP 202
-{"id":1} HTTP 202
-GET /api/orders (step 5):
+          <t>Step 1 (Send an empty JSON object):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:54:58 GMT
+Content-Length: 9
+{"id":1}
+Step 2 (Send Ann's order without order_id):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:54:58 GMT
+Content-Length: 9
+{"id":1}
+Step 3 (Send Bob's order without order_id):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:54:58 GMT
+Content-Length: 9
+{"id":1}
+Step 5 (List orders):
 {
     "limit": 50,
     "offset": 0,
@@ -1320,13 +1238,13 @@
             "notes": "",
             "total": 0,
             "status": "dispatched",
-            "ready_at": "2026-09-27 20:28:09",
-            "created_at": "2026-09-27 20:28:09",
-            "updated_at": "2026-09-27 20:28:10"
+            "ready_at": "2026-09-28 03:54:58",
+            "created_at": "2026-09-28 03:54:58",
+            "updated_at": "2026-09-28 03:54:59"
         }
     ]
 }
-GET /api/orders/1/events (step 6):
+Step 6 (Show the history of order 1):
 {
     "events": [
         {
@@ -1334,7 +1252,7 @@
             "order_id": 1,
             "kind": "received",
             "detail": {},
-            "created_at": "2026-09-27 20:28:09"
+            "created_at": "2026-09-28 03:54:58"
         },
         {
             "id": 2,
@@ -1351,7 +1269,7 @@
                 ],
                 "notes": ""
             },
-            "created_at": "2026-09-27 20:28:09"
+            "created_at": "2026-09-28 03:54:58"
         },
         {
             "id": 3,
@@ -1368,36 +1286,36 @@
                 ],
                 "notes": ""
             },
-            "created_at": "2026-09-27 20:28:09"
+            "created_at": "2026-09-28 03:54:58"
         },
         {
             "id": 4,
             "order_id": 1,
             "kind": "dispatched",
             "detail": {
-                "dispatch_id": "06fba4c254a0b5ac",
+                "dispatch_id": "dfd57ff0acce6143",
                 "order_id": 1,
                 "external_ref": "webhook:",
                 "source": "webhook",
                 "station": "assembly-1",
                 "customer": " ",
                 "items": null,
-                "dispatch_at": "2026-09-27T20:28:10Z"
+                "dispatch_at": "2026-09-28T03:54:59Z"
             },
-            "created_at": "2026-09-27 20:28:10"
+            "created_at": "2026-09-28 03:54:59"
         }
     ]
 }
-data/robot_dispatch.jsonl (step 7):
-{"dispatch_id":"06fba4c254a0b5ac","order_id":1,"external_ref":"webhook:","source":"webhook","station":"assembly-1","customer":" ","items":null,"dispatch_at":"2026-09-27T20:28:10Z"}
-OrderHub log:
-2026/09/27 13:28:08 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 13:28:08 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 13:28:08 poller: polling http://localhost:8090 every 2s
-2026/09/27 13:28:09 POST /webhooks/orders 0s
-2026/09/27 13:28:09 POST /webhooks/orders 0s
-2026/09/27 13:28:09 POST /webhooks/orders 0s
-2026/09/27 13:28:10 dispatch: sent 1 orders</t>
+Step 7 (Show what the robot received):
+{"dispatch_id":"dfd57ff0acce6143","order_id":1,"external_ref":"webhook:","source":"webhook","station":"assembly-1","customer":" ","items":null,"dispatch_at":"2026-09-28T03:54:59Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:54:57 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:54:57 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:54:57 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:54:58 POST /webhooks/orders 0s
+2026/09/27 20:54:58 POST /webhooks/orders 0s
+2026/09/27 20:54:58 POST /webhooks/orders 0s
+2026/09/27 20:54:59 dispatch: sent 1 orders</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -1420,11 +1338,6 @@
 - Valid orders must still be accepted: python -m pytest -m smoke.</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_webhook.py::test_webhook_with_missing_fields_is_rejected</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="150" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1439,66 +1352,46 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>tests/test_partner_api.py::test_order_in_the_same_window_as_a_500_is_not_lost</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Partner API polling</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>When one poll of the partner API gets a 500, every order that happened upstream in that poll's time window is never picked up. The next poll starts after the failed window instead of retrying it. The orders are never stored and never made, and nothing is logged about them.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>- README, Pipelines, Partner API: "The API sometimes fails with a 500, and a retry of the same request succeeds. Nothing that happens upstream may be lost."
 - README, Mock partner API: "An enqueued response with a non-200 response is a transient upstream failure. The first poll whose window covers it gets that failure back. Retrying the same time_since succeeds and returns everything else enqueued in that window."</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
-- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
-- No other traffic is sent to OrderHub or the mock while reproducing.
-Steps:
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. make run also starts the mock partner API on port 8090.
 1. Enqueue a 500 and an order on the mock, one right after the other (within 2 seconds, so both land in the same poll window). Run both lines together:
 curl -s -X POST localhost:8090/enqueue -d '{"response":500,"error":"Internal server error"}'
 curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-5005-1":{"order":5005,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"}}}'
-2. Confirm the mock recorded both: curl -s localhost:8090/status
+2. Confirm the mock recorded both:
+curl -s localhost:8090/status
 3. Wait 10 seconds (5 poll cycles).
-4. List partner orders: curl -s 'localhost:8080/api/orders?source=api' | python3 -m json.tool
-5. Control: enqueue a second order on its own, wait 4 seconds, and list again:
+4. List partner orders:
+curl -s 'localhost:8080/api/orders?source=api' | python3 -m json.tool
+5. Control: enqueue a second order on its own, then list partner orders again 4 seconds later:
 curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-5006-1":{"order":5006,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"}}}'
+sleep 4
 curl -s 'localhost:8080/api/orders?source=api' | python3 -m json.tool
 6. Look at the OrderHub log in the make run terminal.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Failure response:
-{"response": 500, "error": "Internal server error"}
-Partner order 5005, sent in the same poll window:
-{
-  "response": 200,
-  "data": {
-    "i-5005-1": {"order": 5005, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"}
-  }
-}
-Control order 5006, sent later on its own:
-{
-  "response": 200,
-  "data": {
-    "i-5006-1": {"order": 5006, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"}
-  }
-}</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1519,19 +1412,19 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Mock responses and GET localhost:8090/status (steps 1 and 2):
-enqueued at 2026-09-27T21:55:10.524409898Z
-enqueued at 2026-09-27T21:55:10.531793697Z
+          <t>Step 1 (Enqueue a 500 and an order on the mock, one right after the other (within 2 seconds, so both land in the same poll window). Run both lines together):
+enqueued at 2026-09-28T03:55:04.8502851Z
+enqueued at 2026-09-28T03:55:04.855986809Z
+Step 2 (Confirm the mock recorded both):
 {"enqueued":2,"failures":1}
-GET /api/orders?source=api after 10 seconds (step 4):
+Step 4 (List partner orders):
 {
     "limit": 50,
     "offset": 0,
     "orders": []
 }
-Control order 5006 enqueued on its own (step 5):
-enqueued at 2026-09-27T21:55:20.588867144Z
-GET /api/orders?source=api (step 5):
+Step 5 (Control):
+enqueued at 2026-09-28T03:55:14.903031824Z
 {
     "limit": 50,
     "offset": 0,
@@ -1556,18 +1449,18 @@
             "notes": "",
             "total": 4.25,
             "status": "dispatched",
-            "ready_at": "2026-09-27 21:55:20",
-            "created_at": "2026-09-27 21:55:20",
-            "updated_at": "2026-09-27 21:55:22"
+            "ready_at": "2026-09-28 03:55:15",
+            "created_at": "2026-09-28 03:55:15",
+            "updated_at": "2026-09-28 03:55:16"
         }
     ]
 }
-OrderHub log:
-2026/09/27 14:55:08 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 14:55:08 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 14:55:08 poller: polling http://localhost:8090 every 2s
-2026/09/27 14:55:10 poller: upstream returned 500: Internal server error
-2026/09/27 14:55:22 dispatch: sent 1 orders</t>
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:55:03 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:55:03 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:55:03 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:55:05 poller: upstream returned 500: Internal server error
+2026/09/27 20:55:16 dispatch: sent 1 orders</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1590,11 +1483,6 @@
 - tests/test_partner_api.py::test_polling_recovers_after_a_500 must still pass.</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_partner_api.py::test_order_in_the_same_window_as_a_500_is_not_lost</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="150" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -1609,63 +1497,45 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>tests/test_partner_api.py::test_status_update_for_one_item_keeps_the_other_items</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Partner API merging</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>The partner API only sends the items that changed. When an update arrives for one item of a two-item order, OrderHub replaces the order's item list with just that one item. The other item disappears from the order and the total drops to the price of the updated item.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>- README, Pipelines, Partner API: "The response contains every item that changed since time_since ... A response only contains the items that changed."
 - README, Payload formats, Partner API: "Each key in data is an item id. Items belong to orders via order."</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
-- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
-- No other traffic is sent to OrderHub or the mock while reproducing.
-Steps:
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. make run also starts the mock partner API on port 8090.
 1. Enqueue partner order 6006 with two items:
 curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-6006-1":{"order":6006,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"},"i-6006-2":{"order":6006,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"ordered"}}}'
-2. Wait 4 seconds, then show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+2. Wait 4 seconds, then show the order:
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
 3. Enqueue a status update for Cold brew only (processing):
 curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-6006-1":{"order":6006,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"processing"}}}'
-4. Wait 4 seconds, then show the order again: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
-5. Show its history: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
-6. Show what the robot received: cat data/robot_dispatch.jsonl</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Order 6006, first response:
-{
-  "response": 200,
-  "data": {
-    "i-6006-1": {"order": 6006, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"},
-    "i-6006-2": {"order": 6006, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "ordered"}
-  }
-}
-Update for one item:
-{
-  "response": 200,
-  "data": {
-    "i-6006-1": {"order": 6006, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "processing"}
-  }
-}</t>
+4. Wait 4 seconds, then show the order again:
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+5. Show its history:
+curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+6. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1685,7 +1555,9 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>GET /api/orders/1 before the update (step 2):
+          <t>Step 1 (Enqueue partner order 6006 with two items):
+enqueued at 2026-09-28T03:55:21.98462479Z
+Step 2 (Wait 4 seconds, then show the order):
 {
     "id": 1,
     "source": "api",
@@ -1713,12 +1585,13 @@
     "notes": "",
     "total": 15.75,
     "status": "dispatched",
-    "ready_at": "2026-09-27 21:55:27",
-    "created_at": "2026-09-27 21:55:27",
-    "updated_at": "2026-09-27 21:55:28"
+    "ready_at": "2026-09-28 03:55:22",
+    "created_at": "2026-09-28 03:55:22",
+    "updated_at": "2026-09-28 03:55:23"
 }
-enqueued at 2026-09-27T21:55:30.723173904Z
-GET /api/orders/1 after the update (step 4):
+Step 3 (Enqueue a status update for Cold brew only (processing)):
+enqueued at 2026-09-28T03:55:26.028974262Z
+Step 4 (Wait 4 seconds, then show the order again):
 {
     "id": 1,
     "source": "api",
@@ -1739,11 +1612,11 @@
     "notes": "",
     "total": 4.25,
     "status": "dispatched",
-    "ready_at": "2026-09-27 21:55:27",
-    "created_at": "2026-09-27 21:55:27",
-    "updated_at": "2026-09-27 21:55:31"
+    "ready_at": "2026-09-28 03:55:22",
+    "created_at": "2026-09-28 03:55:22",
+    "updated_at": "2026-09-28 03:55:26"
 }
-GET /api/orders/1/events (step 5):
+Step 5 (Show its history):
 {
     "events": [
         {
@@ -1769,14 +1642,14 @@
                 ],
                 "order": 6006
             },
-            "created_at": "2026-09-27 21:55:27"
+            "created_at": "2026-09-28 03:55:22"
         },
         {
             "id": 2,
             "order_id": 1,
             "kind": "dispatched",
             "detail": {
-                "dispatch_id": "ab4ecf0d4cc3b632",
+                "dispatch_id": "176f976dad44390a",
                 "order_id": 1,
                 "external_ref": "api:6006",
                 "source": "api",
@@ -1794,9 +1667,9 @@
                         "qty": 1
                     }
                 ],
-                "dispatch_at": "2026-09-27T21:55:28Z"
+                "dispatch_at": "2026-09-28T03:55:23Z"
             },
-            "created_at": "2026-09-27 21:55:28"
+            "created_at": "2026-09-28 03:55:23"
         },
         {
             "id": 3,
@@ -1807,17 +1680,17 @@
                     "Cold brew": "processing"
                 }
             },
-            "created_at": "2026-09-27 21:55:31"
+            "created_at": "2026-09-28 03:55:26"
         }
     ]
 }
-data/robot_dispatch.jsonl (step 6):
-{"dispatch_id":"ab4ecf0d4cc3b632","order_id":1,"external_ref":"api:6006","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-27T21:55:28Z"}
-OrderHub log:
-2026/09/27 14:55:25 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 14:55:25 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 14:55:25 poller: polling http://localhost:8090 every 2s
-2026/09/27 14:55:28 dispatch: sent 1 orders</t>
+Step 6 (Show what the robot received):
+{"dispatch_id":"176f976dad44390a","order_id":1,"external_ref":"api:6006","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-28T03:55:23Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:55:20 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:55:20 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:55:20 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:55:23 dispatch: sent 1 orders</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1839,11 +1712,6 @@
 - python -m pytest tests/test_partner_api.py -k keeps_the_other_items must pass (remove the xfail marker once it reports XPASS(strict)).</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_partner_api.py::test_status_update_for_one_item_keeps_the_other_items</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="150" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1858,63 +1726,45 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>tests/test_partner_api.py::test_cancelling_one_item_does_not_cancel_the_order</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Partner API merging, cancellation</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>When the partner API cancels one item of a two-item order, OrderHub cancels the whole order. The order had already been sent to the robot, so it now shows as cancelled although the food was made.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>- README, Payload formats, Partner API: "An order whose items are all cancelled is cancelled." So an order with some items cancelled is not cancelled.
 - README, Order lifecycle: "Once an order is dispatched, the robot is already building it, so it can no longer be cancelled."</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
-- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
-- No other traffic is sent to OrderHub or the mock while reproducing.
-Steps:
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. make run also starts the mock partner API on port 8090.
 1. Enqueue partner order 7007 with two items:
 curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-7007-1":{"order":7007,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"},"i-7007-2":{"order":7007,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"ordered"}}}'
-2. Wait 4 seconds, then show the order (it is dispatched): curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+2. Wait 4 seconds, then show the order (it is dispatched):
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
 3. Enqueue a cancel for Blueberry pancakes only:
 curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-7007-2":{"order":7007,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"cancelled"}}}'
-4. Wait 4 seconds, then show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
-5. Show its history: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
-6. Show what the robot received: cat data/robot_dispatch.jsonl</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Order 7007, first response:
-{
-  "response": 200,
-  "data": {
-    "i-7007-1": {"order": 7007, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"},
-    "i-7007-2": {"order": 7007, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "ordered"}
-  }
-}
-Cancel for one item:
-{
-  "response": 200,
-  "data": {
-    "i-7007-2": {"order": 7007, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "cancelled"}
-  }
-}</t>
+4. Wait 4 seconds, then show the order:
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+5. Show its history:
+curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+6. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1934,7 +1784,9 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>GET /api/orders/1 before the cancel (step 2):
+          <t>Step 1 (Enqueue partner order 7007 with two items):
+enqueued at 2026-09-28T03:55:33.164707295Z
+Step 2 (Wait 4 seconds, then show the order (it is dispatched)):
 {
     "id": 1,
     "source": "api",
@@ -1962,12 +1814,13 @@
     "notes": "",
     "total": 15.75,
     "status": "dispatched",
-    "ready_at": "2026-09-27 21:55:37",
-    "created_at": "2026-09-27 21:55:37",
-    "updated_at": "2026-09-27 21:55:38"
+    "ready_at": "2026-09-28 03:55:33",
+    "created_at": "2026-09-28 03:55:33",
+    "updated_at": "2026-09-28 03:55:34"
 }
-enqueued at 2026-09-27T21:55:40.900354587Z
-GET /api/orders/1 after the cancel (step 4):
+Step 3 (Enqueue a cancel for Blueberry pancakes only):
+enqueued at 2026-09-28T03:55:37.216381235Z
+Step 4 (Wait 4 seconds, then show the order):
 {
     "id": 1,
     "source": "api",
@@ -1988,11 +1841,11 @@
     "notes": "",
     "total": 11.5,
     "status": "cancelled",
-    "ready_at": "2026-09-27 21:55:37",
-    "created_at": "2026-09-27 21:55:37",
-    "updated_at": "2026-09-27 21:55:41"
+    "ready_at": "2026-09-28 03:55:33",
+    "created_at": "2026-09-28 03:55:33",
+    "updated_at": "2026-09-28 03:55:37"
 }
-GET /api/orders/1/events (step 5):
+Step 5 (Show its history):
 {
     "events": [
         {
@@ -2018,14 +1871,14 @@
                 ],
                 "order": 7007
             },
-            "created_at": "2026-09-27 21:55:37"
+            "created_at": "2026-09-28 03:55:33"
         },
         {
             "id": 2,
             "order_id": 1,
             "kind": "dispatched",
             "detail": {
-                "dispatch_id": "7cc3b56bcb111c81",
+                "dispatch_id": "e45207513ee8e186",
                 "order_id": 1,
                 "external_ref": "api:7007",
                 "source": "api",
@@ -2043,9 +1896,9 @@
                         "qty": 1
                     }
                 ],
-                "dispatch_at": "2026-09-27T21:55:38Z"
+                "dispatch_at": "2026-09-28T03:55:34Z"
             },
-            "created_at": "2026-09-27 21:55:38"
+            "created_at": "2026-09-28 03:55:34"
         },
         {
             "id": 3,
@@ -2056,7 +1909,7 @@
                     "Blueberry pancakes": "cancelled"
                 }
             },
-            "created_at": "2026-09-27 21:55:41"
+            "created_at": "2026-09-28 03:55:37"
         },
         {
             "id": 4,
@@ -2065,17 +1918,17 @@
             "detail": {
                 "by": "partner-api"
             },
-            "created_at": "2026-09-27 21:55:41"
+            "created_at": "2026-09-28 03:55:37"
         }
     ]
 }
-data/robot_dispatch.jsonl (step 6):
-{"dispatch_id":"7cc3b56bcb111c81","order_id":1,"external_ref":"api:7007","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-27T21:55:38Z"}
-OrderHub log:
-2026/09/27 14:55:35 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 14:55:35 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 14:55:35 poller: polling http://localhost:8090 every 2s
-2026/09/27 14:55:38 dispatch: sent 1 orders</t>
+Step 6 (Show what the robot received):
+{"dispatch_id":"e45207513ee8e186","order_id":1,"external_ref":"api:7007","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-28T03:55:34Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:55:31 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:55:31 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:55:31 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:55:34 dispatch: sent 1 orders</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -2098,11 +1951,6 @@
 - python -m pytest tests/test_partner_api.py -k cancelling_one_item must pass (remove the xfail marker once it reports XPASS(strict)).</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_partner_api.py::test_cancelling_one_item_does_not_cancel_the_order</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="150" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -2117,54 +1965,43 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>tests/test_partner_api.py::test_order_that_arrives_fully_cancelled_is_never_dispatched</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Partner API merging, cancellation</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>If OrderHub first sees a partner order when all its items are already cancelled (the customer cancelled before the next poll), it creates the order as queued and sends it to the robot. The cancelled status of the items is ignored.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>- README, Payload formats, Partner API: "An order whose items are all cancelled is cancelled."
 - README, Order lifecycle: "A cancelled order is never dispatched."
 - The poll interval is 2 seconds and the mock merges everything in a window into one response, so an order and its cancellation can arrive in the same poll.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
-- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
-- No other traffic is sent to OrderHub or the mock while reproducing.
-Steps:
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. make run also starts the mock partner API on port 8090.
 1. Enqueue partner order 8008 with both items already cancelled:
 curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-8008-1":{"order":8008,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"cancelled"},"i-8008-2":{"order":8008,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"cancelled"}}}'
 2. Wait 5 seconds.
-3. Show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
-4. Show its history: curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
-5. Show what the robot received: cat data/robot_dispatch.jsonl</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>{
-  "response": 200,
-  "data": {
-    "i-8008-1": {"order": 8008, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "cancelled"},
-    "i-8008-2": {"order": 8008, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "cancelled"}
-  }
-}</t>
+3. Show the order:
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+4. Show its history:
+curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+5. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -2182,7 +2019,9 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>GET /api/orders/1 (step 3):
+          <t>Step 1 (Enqueue partner order 8008 with both items already cancelled):
+enqueued at 2026-09-28T03:55:44.332946241Z
+Step 3 (Show the order):
 {
     "id": 1,
     "source": "api",
@@ -2210,11 +2049,11 @@
     "notes": "",
     "total": 15.75,
     "status": "dispatched",
-    "ready_at": "2026-09-27 21:55:47",
-    "created_at": "2026-09-27 21:55:47",
-    "updated_at": "2026-09-27 21:55:48"
+    "ready_at": "2026-09-28 03:55:44",
+    "created_at": "2026-09-28 03:55:44",
+    "updated_at": "2026-09-28 03:55:45"
 }
-GET /api/orders/1/events (step 4):
+Step 4 (Show its history):
 {
     "events": [
         {
@@ -2240,14 +2079,14 @@
                 ],
                 "order": 8008
             },
-            "created_at": "2026-09-27 21:55:47"
+            "created_at": "2026-09-28 03:55:44"
         },
         {
             "id": 2,
             "order_id": 1,
             "kind": "dispatched",
             "detail": {
-                "dispatch_id": "69ca66b7ed464e31",
+                "dispatch_id": "b33225de99557105",
                 "order_id": 1,
                 "external_ref": "api:8008",
                 "source": "api",
@@ -2265,19 +2104,19 @@
                         "qty": 1
                     }
                 ],
-                "dispatch_at": "2026-09-27T21:55:48Z"
+                "dispatch_at": "2026-09-28T03:55:45Z"
             },
-            "created_at": "2026-09-27 21:55:48"
+            "created_at": "2026-09-28 03:55:45"
         }
     ]
 }
-data/robot_dispatch.jsonl (step 5):
-{"dispatch_id":"69ca66b7ed464e31","order_id":1,"external_ref":"api:8008","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-27T21:55:48Z"}
-OrderHub log:
-2026/09/27 14:55:45 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 14:55:45 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 14:55:45 poller: polling http://localhost:8090 every 2s
-2026/09/27 14:55:48 dispatch: sent 1 orders</t>
+Step 5 (Show what the robot received):
+{"dispatch_id":"b33225de99557105","order_id":1,"external_ref":"api:8008","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-28T03:55:45Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:55:42 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:55:42 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:55:42 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:55:45 dispatch: sent 1 orders</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -2299,11 +2138,6 @@
 - python -m pytest tests/test_partner_api.py -k fully_cancelled must pass (remove the xfail marker once it reports XPASS(strict)).</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_partner_api.py::test_order_that_arrives_fully_cancelled_is_never_dispatched</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="150" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -2318,52 +2152,40 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>tests/test_partner_api.py::test_cancelled_item_is_not_sent_to_the_robot</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Partner API merging, robot payload</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>A partner order with one ordered item and one cancelled item is sent to the robot with both items. The robot makes the cancelled item.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>- README, Payload formats, Partner API: item status "moves through ordered, processing, with_courier, and delivered, or becomes cancelled".
 - README, Order lifecycle: "A cancelled order is never dispatched." The spec does not spell out item-level cancellation, but making an item the customer cancelled contradicts the intent. Question for the team to confirm.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Environment:
-- OrderHub from orderhub.zip, built with make build, started with make run (default flags: site time zone America/New_York, partner API poll every 2s, dispatcher every 1s, simulated robot writing to data/robot_dispatch.jsonl). make run also starts the mock partner API on port 8090.
-- Also reproduced by the automated test, which starts its own OrderHub and mock on a fresh database and captures robot dispatches over HTTP (-robot-url).
-- Client tools: curl, and python3 -m json.tool only to pretty-print JSON.
-Before you start:
-- OrderHub is stopped (Ctrl-C in the make run terminal).
-- In the orderhub folder, run make reset to delete the database and robot log, then make run. This also restarts the mock partner API with nothing enqueued.
-- No other traffic is sent to OrderHub or the mock while reproducing.
-Steps:
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. make run also starts the mock partner API on port 8090.
 1. Enqueue partner order 9009 with Cold brew ordered and Blueberry pancakes cancelled:
 curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-9009-1":{"order":9009,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"},"i-9009-2":{"order":9009,"name":"Blueberry pancakes","category":"Breakfast","price":11.5,"status":"cancelled"}}}'
 2. Wait 5 seconds.
-3. Show the order: curl -s localhost:8080/api/orders/1 | python3 -m json.tool
-4. Show what the robot received: cat data/robot_dispatch.jsonl</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>{
-  "response": 200,
-  "data": {
-    "i-9009-1": {"order": 9009, "name": "Cold brew", "category": "Coffee &amp; Tea", "price": 4.25, "status": "ordered"},
-    "i-9009-2": {"order": 9009, "name": "Blueberry pancakes", "category": "Breakfast", "price": 11.5, "status": "cancelled"}
-  }
-}</t>
+3. Show the order:
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+4. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -2380,7 +2202,9 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>GET /api/orders/1 (step 3):
+          <t>Step 1 (Enqueue partner order 9009 with Cold brew ordered and Blueberry pancakes cancelled):
+enqueued at 2026-09-28T03:55:52.448043692Z
+Step 3 (Show the order):
 {
     "id": 1,
     "source": "api",
@@ -2408,17 +2232,17 @@
     "notes": "",
     "total": 15.75,
     "status": "dispatched",
-    "ready_at": "2026-09-27 21:55:54",
-    "created_at": "2026-09-27 21:55:54",
-    "updated_at": "2026-09-27 21:55:55"
+    "ready_at": "2026-09-28 03:55:52",
+    "created_at": "2026-09-28 03:55:52",
+    "updated_at": "2026-09-28 03:55:53"
 }
-data/robot_dispatch.jsonl (step 4):
-{"dispatch_id":"947dff8a958d0725","order_id":1,"external_ref":"api:9009","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-27T21:55:55Z"}
-OrderHub log:
-2026/09/27 14:55:52 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 14:55:52 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 14:55:52 poller: polling http://localhost:8090 every 2s
-2026/09/27 14:55:55 dispatch: sent 1 orders</t>
+Step 4 (Show what the robot received):
+{"dispatch_id":"bedfb6c5e37e174d","order_id":1,"external_ref":"api:9009","source":"api","station":"assembly-1","customer":" ","items":[{"line":1,"name":"Blueberry pancakes","qty":1},{"line":2,"name":"Cold brew","qty":1}],"dispatch_at":"2026-09-28T03:55:53Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:55:50 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:55:50 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:55:50 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:55:53 dispatch: sent 1 orders</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -2439,26 +2263,674 @@
 - python -m pytest tests/test_partner_api.py -k cancelled_item_is_not_sent must pass (remove the xfail marker once it reports XPASS(strict)).</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>tests/test_partner_api.py::test_cancelled_item_is_not_sent_to_the_robot</t>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>L37-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Orders are sent to the robot more than once during a burst (100 orders became 194 builds)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_dispatch.py::test_burst_at_normal_robot_speed_makes_each_order_once
+tests/test_dispatch.py::test_slow_robot_makes_each_order_once</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Dispatch</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>When more orders are waiting than the robot can accept in one second, the same orders are sent to the robot again on the next dispatcher tick, and again on the one after. With the simulated robot's normal speed, a burst of 100 orders produced 194 builds: 65 orders were made more than once, some three times. The order list and dashboard still show 100 dispatched orders, so the duplicates are only visible at the robot.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>- README, Order lifecycle: "Each order is dispatched to the robot exactly once."
+- README, Pipelines, Webhook: "Traffic is bursty."
+- README, Capacity: "OrderHub must handle 100,000 requests per day, arriving in bursts rather than evenly."
+- README, Design notes: "Dispatch runs on a one-second ticker in the background so a slow robot doesn't block ingest."</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Send a burst of 100 different webhook orders at the same time (each has its own order_id):
+for i in $(seq 1 100); do
+  curl -s -o /dev/null -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d "{\"order_id\":\"burst-$i\",\"order_source\":\"Grubstub\",\"restaurant\":\"Just Pizza\",\"first_name\":\"Guest\",\"last_name\":\"$i\",\"total\":10,\"items\":[\"Margherita pizza\"],\"notes\":\"\"}" &amp;
+done; wait
+2. Wait 10 seconds.
+3. Dashboard counts:
+curl -s localhost:8080/api/stats | python3 -m json.tool
+4. Number of orders the robot received:
+wc -l &lt; data/robot_dispatch.jsonl
+5. Number of orders the robot received more than once:
+grep -o '"order_id":[0-9]*' data/robot_dispatch.jsonl | sort | uniq -c | awk '$1 &gt; 1' | wc -l
+6. Orders the robot received most often:
+grep -o '"order_id":[0-9]*' data/robot_dispatch.jsonl | sort | uniq -c | sort -rn | head -3
+7. For one of those (order 99 in my run), show the robot lines and its history:
+grep '"order_id":99,' data/robot_dispatch.jsonl
+curl -s localhost:8080/api/orders/99/events | python3 -m json.tool</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>- Step 3: 100 orders, all dispatched.
+- Step 4: 100 lines, one per order.
+- Step 5: 0.
+- Step 7: one robot line and one dispatched event per order.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>- Step 3: 100 orders, all dispatched. The dashboard looks correct.
+- Step 4: 194 lines. The robot was asked to build 194 pizzas for 100 orders.
+- Step 5: 65 orders were sent more than once.
+- Step 6: some orders were sent 3 times.
+- Step 7: order 99 reached the robot 3 times, each time with a different dispatch_id, and its history has 3 dispatched events. The robot has no way to tell these are the same order.
+- OrderHub log: "dispatch: sent 100 orders", "sent 29 orders", "sent 65 orders" within about a second.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Send a burst of 100 different webhook orders at the same time (each has its own order_id)):
+(no output)
+Step 3 (Dashboard counts):
+{
+    "by_status": {
+        "dispatched": 100
+    },
+    "by_source": {
+        "webhook": 100
+    },
+    "by_platform": {
+        "Grubstub": 100
+    },
+    "total_orders": 100,
+    "total_events": 294,
+    "last_hour": 100,
+    "refreshed_at": "2026-09-28T03:56:03Z"
+}
+Step 4 (Number of orders the robot received):
+194
+Step 5 (Number of orders the robot received more than once):
+65
+Step 6 (Orders the robot received most often):
+3 "order_id":99
+      3 "order_id":98
+      3 "order_id":97
+Step 7 (For one of those (order 99 in my run), show the robot lines and its history):
+{"dispatch_id":"d1eee0c61302433d","order_id":99,"external_ref":"webhook:burst-82","source":"webhook","station":"assembly-1","customer":"Guest 82","items":[{"line":1,"name":"Margherita pizza","qty":1}],"dispatch_at":"2026-09-28T03:56:03Z"}
+{"dispatch_id":"2679dd4c5b0a852d","order_id":99,"external_ref":"webhook:burst-82","source":"webhook","station":"assembly-1","customer":"Guest 82","items":[{"line":1,"name":"Margherita pizza","qty":1}],"dispatch_at":"2026-09-28T03:56:03Z"}
+{"dispatch_id":"8d8683e258b20e10","order_id":99,"external_ref":"webhook:burst-82","source":"webhook","station":"assembly-1","customer":"Guest 82","items":[{"line":1,"name":"Margherita pizza","qty":1}],"dispatch_at":"2026-09-28T03:56:03Z"}
+{
+    "events": [
+        {
+            "id": 99,
+            "order_id": 99,
+            "kind": "received",
+            "detail": {
+                "order_id": "burst-82",
+                "order_source": "Grubstub",
+                "restaurant": "Just Pizza",
+                "first_name": "Guest",
+                "last_name": "82",
+                "total": 10,
+                "items": [
+                    "Margherita pizza"
+                ],
+                "notes": ""
+            },
+            "created_at": "2026-09-28 03:56:00"
+        },
+        {
+            "id": 288,
+            "order_id": 99,
+            "kind": "dispatched",
+            "detail": {
+                "dispatch_id": "d1eee0c61302433d",
+                "order_id": 99,
+                "external_ref": "webhook:burst-82",
+                "source": "webhook",
+                "station": "assembly-1",
+                "customer": "Guest 82",
+                "items": [
+                    {
+                        "line": 1,
+                        "name": "Margherita pizza",
+                        "qty": 1
+                    }
+                ],
+                "dispatch_at": "2026-09-28T03:56:03Z"
+            },
+            "created_at": "2026-09-28 03:56:03"
+        },
+        {
+            "id": 289,
+            "order_id": 99,
+            "kind": "dispatched",
+            "detail": {
+                "dispatch_id": "2679dd4c5b0a852d",
+                "order_id": 99,
+                "external_ref": "webhook:burst-82",
+                "source": "webhook",
+                "station": "assembly-1",
+                "customer": "Guest 82",
+                "items": [
+                    {
+                        "line": 1,
+                        "name": "Margherita pizza",
+                        "qty": 1
+                    }
+                ],
+                "dispatch_at": "2026-09-28T03:56:03Z"
+            },
+            "created_at": "2026-09-28 03:56:03"
+        },
+        {
+            "id": 292,
+            "order_id": 99,
+            "kind": "dispatched",
+            "detail": {
+                "dispatch_id": "8d8683e258b20e10",
+                "order_id": 99,
+                "external_ref": "webhook:burst-82",
+                "source": "webhook",
+                "station": "assembly-1",
+                "customer": "Guest 82",
+                "items": [
+                    {
+                        "line": 1,
+                        "name": "Margherita pizza",
+                        "qty": 1
+                    }
+                ],
+                "dispatch_at": "2026-09-28T03:56:03Z"
+            },
+            "created_at": "2026-09-28 03:56:03"
+        }
+    ]
+}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:55:59 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:55:59 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:55:59 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:56:03 dispatch: sent 100 orders
+2026/09/27 20:56:03 dispatch: sent 29 orders
+2026/09/27 20:56:03 dispatch: sent 65 orders
+(100 lines "POST /webhooks/orders" not shown)
+Automated test, robot at 30 ms per order, burst of 60: 29 of 60 orders made twice, in 3 of 3 runs.
+Earlier run with the test receiver at 30 ms: burst of 20 made 20 builds (no duplicates); 50 made 69; 100 made 211 (69 orders duplicated, up to 4 times).</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>- Food is made two or three times for one order: wasted food, robot time and kitchen capacity, exactly during the busiest periods.
+- Duplicates grow with burst size: no duplicates at 20 orders, 19 at 50, 60+ at 100. Bursts are part of the spec, so this happens in normal operation.
+- Every duplicate slows the robot further, which makes the next batch slower and creates more duplicates.
+- Nothing in the UI, the order list or the dashboard shows it. Only the robot and the event history see it.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>- The exact numbers vary a little between runs (188, 194, 195 and 197 builds in my runs of these steps), but the robot always received well over 100.
+- Black-box inference: the dispatcher seems to start a new batch every second without waiting for the previous one. An order stays queued until its batch reaches it, so the next batch picks it up again.
+- Each attempt gets a new dispatch_id, so the robot cannot de-duplicate on its side.
+- The same happens with a slow robot: with 1.5 seconds per order, 5 orders became 26 builds (one order 8 times). See tests/test_dispatch.py::test_slow_robot_makes_each_order_once.
+- The load test will measure how often this happens at 100,000 requests a day.
+- Related: L37-012 (same timing window lets a cancel be undone).</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above several times. Step 4 must be exactly 100 and step 5 must be 0 every time.
+- Repeat with 300 orders.
+- python -m pytest tests/test_dispatch.py -k "burst or slow_robot" must pass (remove the xfail markers once they report XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>L37-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>An order the robot is already building can be cancelled through the API</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_dispatch.py::test_dispatched_order_cannot_be_cancelled</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Cancellation, operator API</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/orders/{id}/cancel accepts a cancel for an order that was already dispatched. It returns 200 and the order becomes cancelled, although the robot is already building it. The UI correctly disables the checkbox for dispatched orders, but the API does not enforce the rule.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>- README, Order lifecycle: "Once an order is dispatched, the robot is already building it, so it can no longer be cancelled."
+- README, Order lifecycle diagram: only scheduled or queued orders can be cancelled.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Send an order:
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"1111","order_source":"Grubstub","restaurant":"Just Pizza","first_name":"Ada","last_name":"Park","total":24.5,"items":["Margherita pizza","Garlic knots"],"notes":""}'
+2. Wait 3 seconds, then show it (dispatched):
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool
+3. Cancel it through the operator API:
+curl -si -X POST localhost:8080/api/orders/1/cancel
+4. Show its history:
+curl -s localhost:8080/api/orders/1/events | python3 -m json.tool
+5. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>- Step 3 is refused with an error (for example 409 Conflict) saying the order was already dispatched.
+- The order stays dispatched, and the history has no cancelled event.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2: dispatched.
+- Step 3: HTTP 200, and the returned order has status cancelled.
+- Step 4: received, dispatched, then cancelled by operator.
+- Step 5: the robot received the order before the cancel. It was made, but OrderHub now says it was cancelled.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Send an order):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:56:14 GMT
+Content-Length: 9
+{"id":1}
+Step 2 (Wait 3 seconds, then show it (dispatched)):
+{
+    "id": 1,
+    "source": "webhook",
+    "external_id": "1111",
+    "platform": "Grubstub",
+    "restaurant": "Just Pizza",
+    "customer_first": "Ada",
+    "customer_last": "Park",
+    "items": [
+        {
+            "name": "Margherita pizza"
+        },
+        {
+            "name": "Garlic knots"
+        }
+    ],
+    "notes": "",
+    "total": 24.5,
+    "status": "dispatched",
+    "ready_at": "2026-09-28 03:56:14",
+    "created_at": "2026-09-28 03:56:14",
+    "updated_at": "2026-09-28 03:56:14"
+}
+Step 3 (Cancel it through the operator API):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:56:17 GMT
+Content-Length: 353
+{"id":1,"source":"webhook","external_id":"1111","platform":"Grubstub","restaurant":"Just Pizza","customer_first":"Ada","customer_last":"Park","items":[{"name":"Margherita pizza"},{"name":"Garlic knots"}],"notes":"","total":24.5,"status":"cancelled","ready_at":"2026-09-28 03:56:14","created_at":"2026-09-28 03:56:14","updated_at":"2026-09-28 03:56:17"}
+Step 4 (Show its history):
+{
+    "events": [
+        {
+            "id": 1,
+            "order_id": 1,
+            "kind": "received",
+            "detail": {
+                "order_id": "1111",
+                "order_source": "Grubstub",
+                "restaurant": "Just Pizza",
+                "first_name": "Ada",
+                "last_name": "Park",
+                "total": 24.5,
+                "items": [
+                    "Margherita pizza",
+                    "Garlic knots"
+                ],
+                "notes": ""
+            },
+            "created_at": "2026-09-28 03:56:14"
+        },
+        {
+            "id": 2,
+            "order_id": 1,
+            "kind": "dispatched",
+            "detail": {
+                "dispatch_id": "dc68be315ee0c473",
+                "order_id": 1,
+                "external_ref": "webhook:1111",
+                "source": "webhook",
+                "station": "assembly-1",
+                "customer": "Ada Park",
+                "items": [
+                    {
+                        "line": 1,
+                        "name": "Margherita pizza",
+                        "qty": 1
+                    },
+                    {
+                        "line": 2,
+                        "name": "Garlic knots",
+                        "qty": 1
+                    }
+                ],
+                "dispatch_at": "2026-09-28T03:56:14Z"
+            },
+            "created_at": "2026-09-28 03:56:14"
+        },
+        {
+            "id": 3,
+            "order_id": 1,
+            "kind": "cancelled",
+            "detail": {
+                "by": "operator"
+            },
+            "created_at": "2026-09-28 03:56:17"
+        }
+    ]
+}
+Step 5 (Show what the robot received):
+{"dispatch_id":"dc68be315ee0c473","order_id":1,"external_ref":"webhook:1111","source":"webhook","station":"assembly-1","customer":"Ada Park","items":[{"line":1,"name":"Margherita pizza","qty":1},{"line":2,"name":"Garlic knots","qty":1}],"dispatch_at":"2026-09-28T03:56:14Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:56:12 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:56:12 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:56:12 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:56:14 POST /webhooks/orders 1ms
+2026/09/27 20:56:14 dispatch: sent 1 orders
+2026/09/27 20:56:17 POST /api/orders/1/cancel 0s</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>- OrderHub's records say the order was cancelled while the food was made. Support may refund it or tell the customer it isn't coming.
+- Anything besides the UI that uses the API (scripts, other tools, a future UI change) can cancel dispatched orders.
+- The same thing happens through upstream cancels: see L37-007 (partner API).</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>- The UI disables the checkbox for dispatched orders, which is correct. The rule has to be enforced by the API too, not only by the UI.
+- Related: L37-007, L37-012.</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- Check the same through the UI: dispatched orders cannot be selected.
+- python -m pytest tests/test_dispatch.py -k dispatched_order_cannot_be_cancelled must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>L37-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>A cancel accepted while an order is waiting to be sent is undone, and the order is made</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_dispatch.py::test_cancel_while_the_robot_is_receiving_the_order_is_refused</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Cancellation, dispatch</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>During a burst, an operator cancels an order that is still queued. OrderHub answers 200 with status cancelled. About two seconds later the dispatcher sends the order to the robot anyway and changes its status back to dispatched. The operator was told the order is cancelled; the robot makes it.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>- README, Order lifecycle: "scheduled or queued orders can be cancelled by an operator or upstream" and "A cancelled order is never dispatched."</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Send a burst of 100 orders so the dispatcher has a backlog:
+for i in $(seq 1 100); do
+  curl -s -o /dev/null -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d "{\"order_id\":\"burst-$i\",\"order_source\":\"Grubstub\",\"restaurant\":\"Just Pizza\",\"first_name\":\"Guest\",\"last_name\":\"$i\",\"total\":10,\"items\":[\"Margherita pizza\"],\"notes\":\"\"}" &amp;
+done; wait
+2. Wait 1 second, so the dispatcher has started sending the burst. Then find the newest order (it is still queued):
+curl -s 'localhost:8080/api/orders?limit=1' | python3 -m json.tool
+3. Cancel it right away (order 100 in my run):
+curl -si -X POST localhost:8080/api/orders/100/cancel
+4. Wait 10 seconds.
+5. Show the order:
+curl -s localhost:8080/api/orders/100 | python3 -m json.tool
+6. Show its history:
+curl -s localhost:8080/api/orders/100/events | python3 -m json.tool
+7. Count how often the robot received it:
+grep -c '"order_id":100,' data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Either:
+- the cancel is accepted, the order stays cancelled, and the robot never receives it (step 7 prints 0), or
+- the cancel is refused because the order is already being sent.
+It must never answer "cancelled" and then make the order.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2: order 100 is queued.
+- Step 3: HTTP 200, status cancelled.
+- Step 5: status dispatched.
+- Step 6: received, cancelled, then dispatched two seconds later.
+- Step 7: the robot received the order.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Send a burst of 100 orders so the dispatcher has a backlog):
+(no output)
+Step 2 (Wait 1 second, so the dispatcher has started sending the burst. Then find the newest order (it is still queued)):
+{
+    "limit": 1,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 100,
+            "source": "webhook",
+            "external_id": "burst-91",
+            "platform": "Grubstub",
+            "restaurant": "Just Pizza",
+            "customer_first": "Guest",
+            "customer_last": "91",
+            "items": [
+                {
+                    "name": "Margherita pizza"
+                }
+            ],
+            "notes": "",
+            "total": 10,
+            "status": "queued",
+            "ready_at": "2026-09-28 03:56:20",
+            "created_at": "2026-09-28 03:56:20",
+            "updated_at": "2026-09-28 03:56:20"
+        }
+    ]
+}
+Step 3 (Cancel it right away (order 100 in my run)):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 03:56:21 GMT
+Content-Length: 333
+{"id":100,"source":"webhook","external_id":"burst-91","platform":"Grubstub","restaurant":"Just Pizza","customer_first":"Guest","customer_last":"91","items":[{"name":"Margherita pizza"}],"notes":"","total":10,"status":"cancelled","ready_at":"2026-09-28 03:56:20","created_at":"2026-09-28 03:56:20","updated_at":"2026-09-28 03:56:21"}
+Step 5 (Show the order):
+{
+    "id": 100,
+    "source": "webhook",
+    "external_id": "burst-91",
+    "platform": "Grubstub",
+    "restaurant": "Just Pizza",
+    "customer_first": "Guest",
+    "customer_last": "91",
+    "items": [
+        {
+            "name": "Margherita pizza"
+        }
+    ],
+    "notes": "",
+    "total": 10,
+    "status": "dispatched",
+    "ready_at": "2026-09-28 03:56:20",
+    "created_at": "2026-09-28 03:56:20",
+    "updated_at": "2026-09-28 03:56:23"
+}
+Step 6 (Show its history):
+{
+    "events": [
+        {
+            "id": 100,
+            "order_id": 100,
+            "kind": "received",
+            "detail": {
+                "order_id": "burst-91",
+                "order_source": "Grubstub",
+                "restaurant": "Just Pizza",
+                "first_name": "Guest",
+                "last_name": "91",
+                "total": 10,
+                "items": [
+                    "Margherita pizza"
+                ],
+                "notes": ""
+            },
+            "created_at": "2026-09-28 03:56:20"
+        },
+        {
+            "id": 132,
+            "order_id": 100,
+            "kind": "cancelled",
+            "detail": {
+                "by": "operator"
+            },
+            "created_at": "2026-09-28 03:56:21"
+        },
+        {
+            "id": 290,
+            "order_id": 100,
+            "kind": "dispatched",
+            "detail": {
+                "dispatch_id": "e31ad75cc4a8bc23",
+                "order_id": 100,
+                "external_ref": "webhook:burst-91",
+                "source": "webhook",
+                "station": "assembly-1",
+                "customer": "Guest 91",
+                "items": [
+                    {
+                        "line": 1,
+                        "name": "Margherita pizza",
+                        "qty": 1
+                    }
+                ],
+                "dispatch_at": "2026-09-28T03:56:23Z"
+            },
+            "created_at": "2026-09-28 03:56:23"
+        }
+    ]
+}
+Step 7 (Count how often the robot received it):
+1
+OrderHub log (GET /api lines not shown):
+2026/09/27 20:56:18 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 20:56:18 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 20:56:18 poller: polling http://localhost:8090 every 2s
+2026/09/27 20:56:21 POST /api/orders/100/cancel 1ms
+2026/09/27 20:56:23 dispatch: sent 63 orders
+2026/09/27 20:56:23 dispatch: sent 26 orders
+2026/09/27 20:56:23 dispatch: sent 100 orders
+(100 lines "POST /webhooks/orders" not shown)
+Automated test, robot at 0.8 s per order: the cancel sent while the robot is receiving the order returns 200, and the order ends dispatched, in 3 of 3 runs.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>- A customer's cancellation is confirmed and then ignored. Food is made that nobody wants, and the operator has been told otherwise.
+- The history shows cancelled and then dispatched, so the order looks like it was un-cancelled.
+- The window is widest exactly during bursts, when operators are most likely to be cancelling.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>- Black-box inference: the dispatcher picks up a batch of queued orders at the start of each tick and sends them all, without checking whether any were cancelled in the meantime.
+- Different from L37-011: here the order is still queued when it is cancelled, so fixing L37-011 (refusing cancels of dispatched orders) will not fix this.
+- Related: L37-010, L37-011.</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above several times. Step 7 must print 0 whenever step 3 returned 200.
+- python -m pytest tests/test_dispatch.py -k cancel_while_the_robot must pass (remove the xfail marker once it reports XPASS(strict)).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O10"/>
-  <conditionalFormatting sqref="C2:C1000">
+  <autoFilter ref="A1:N13"/>
+  <conditionalFormatting sqref="D2:D1000">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$C2="Critical"</formula>
+      <formula>$D2="Critical"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$C2="High"</formula>
+      <formula>$D2="High"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>$C2="Medium"</formula>
+      <formula>$D2="Medium"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
-      <formula>$C2="Low"</formula>
+      <formula>$D2="Low"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add csv test, bugs 013-016
</commit_message>
<xml_diff>
--- a/defects/defects.xlsx
+++ b/defects/defects.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2917,8 +2917,653 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="150" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>L37-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Survey meals are scheduled in UTC instead of the kitchen's time zone; -site-tz is ignored</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_csv.py::test_meal_is_scheduled_at_kitchen_local_time (breakfast, lunch, dinner)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Survey CSV, scheduling</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Breakfast, lunch and dinner are scheduled at 8:00, 12:00 and 18:00 UTC instead of 8:00, 12:00 and 18:00 in the kitchen's time zone. With the default America/New_York, every survey order is made 4 hours early (5 hours in winter): breakfast at 4 a.m., lunch at 8 a.m., dinner at 2 p.m. Changing -site-tz makes no difference.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Survey CSV: "meal is breakfast (made at 8:00), lunch (12:00), or dinner (18:00), in the kitchen's local time zone (-site-tz, default America/New_York)."
+- README, Order lifecycle: "Every order has a ready_at: the earliest time it may be sent to the robot ... Survey orders are ready at their meal time."</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Upload a survey export with one order for each meal, all for tomorrow:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nAda,Breakfast,Bagel,,true,breakfast\nAda,Lunch,Soup,,true,lunch\nAda,Dinner,Pasta,,true,dinner\n'
+2. List survey orders and look at ready_at (stored in UTC):
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -m json.tool
+3. Stop OrderHub (Ctrl-C), run make reset, and start it with the kitchen in Los Angeles: ORDERHUB_SITE_TZ=America/Los_Angeles make run
+4. Upload the same export again:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nAda,Breakfast,Bagel,,true,breakfast\nAda,Lunch,Soup,,true,lunch\nAda,Dinner,Pasta,,true,dinner\n'
+5. List survey orders again:
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -m json.tool</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2 (New York, daylight time, UTC-4): ready_at is tomorrow at 12:00:00 (breakfast), 16:00:00 (lunch) and 22:00:00 (dinner) UTC. In winter (UTC-5) it is 13:00, 17:00 and 23:00.
+- Step 5 (Los Angeles, UTC-7): tomorrow at 15:00:00, 19:00:00 and 01:00:00 the day after, UTC.
+- The two runs give different times, because the kitchen is in a different time zone.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>- Step 2: ready_at is tomorrow at 08:00:00, 12:00:00 and 18:00:00 UTC. That is 4:00 a.m., 8:00 a.m. and 2:00 p.m. in New York.
+- Step 5: exactly the same times. The kitchen time zone setting has no effect.
+- The OrderHub log shows it read the setting ("site time zone America/Los_Angeles"), but scheduling doesn't use it.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Upload a survey export with one order for each meal, all for tomorrow):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 04:08:52 GMT
+Content-Length: 82
+{"upload_id":"u1790568532292384113","rows":3,"created":3,"skipped":0,"errors":[]}
+Step 2 (List survey orders and look at ready_at (stored in UTC)):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 3,
+            "source": "csv",
+            "external_id": "u1790568532292384113-4",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Ada",
+            "customer_last": "Dinner",
+            "items": [
+                {
+                    "name": "Pasta"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 18:00:00",
+            "created_at": "2026-09-28 04:08:52",
+            "updated_at": "2026-09-28 04:08:52"
+        },
+        {
+            "id": 2,
+            "source": "csv",
+            "external_id": "u1790568532292384113-3",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Ada",
+            "customer_last": "Lunch",
+            "items": [
+                {
+                    "name": "Soup"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 12:00:00",
+            "created_at": "2026-09-28 04:08:52",
+            "updated_at": "2026-09-28 04:08:52"
+        },
+        {
+            "id": 1,
+            "source": "csv",
+            "external_id": "u1790568532292384113-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Ada",
+            "customer_last": "Breakfast",
+            "items": [
+                {
+                    "name": "Bagel"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 08:00:00",
+            "created_at": "2026-09-28 04:08:52",
+            "updated_at": "2026-09-28 04:08:52"
+        }
+    ]
+}
+Step 3 (Stop OrderHub (Ctrl-C), run make reset, and start it with the kitchen in Los Angeles):
+(restarted OrderHub with ORDERHUB_SITE_TZ=America/Los_Angeles)
+Step 4 (Upload the same export again):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 04:08:54 GMT
+Content-Length: 82
+{"upload_id":"u1790568534382177342","rows":3,"created":3,"skipped":0,"errors":[]}
+Step 5 (List survey orders again):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 3,
+            "source": "csv",
+            "external_id": "u1790568534382177342-4",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Ada",
+            "customer_last": "Dinner",
+            "items": [
+                {
+                    "name": "Pasta"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 18:00:00",
+            "created_at": "2026-09-28 04:08:54",
+            "updated_at": "2026-09-28 04:08:54"
+        },
+        {
+            "id": 2,
+            "source": "csv",
+            "external_id": "u1790568534382177342-3",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Ada",
+            "customer_last": "Lunch",
+            "items": [
+                {
+                    "name": "Soup"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 12:00:00",
+            "created_at": "2026-09-28 04:08:54",
+            "updated_at": "2026-09-28 04:08:54"
+        },
+        {
+            "id": 1,
+            "source": "csv",
+            "external_id": "u1790568534382177342-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Ada",
+            "customer_last": "Breakfast",
+            "items": [
+                {
+                    "name": "Bagel"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 08:00:00",
+            "created_at": "2026-09-28 04:08:54",
+            "updated_at": "2026-09-28 04:08:54"
+        }
+    ]
+}
+OrderHub log (GET /api lines not shown):
+2026/09/27 21:08:50 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 21:08:50 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 21:08:50 poller: polling http://localhost:8090 every 2s
+2026/09/27 21:08:52 csv upload u1790568532292384113: 3 rows, 3 created, 0 skipped, 0 errors
+2026/09/27 21:08:52 POST /uploads/csv 2ms
+2026/09/27 21:08:52 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 21:08:52 orderhub listening on :8080 (site time zone America/Los_Angeles)
+2026/09/27 21:08:52 poller: polling http://localhost:8090 every 2s
+2026/09/27 21:08:54 csv upload u1790568534382177342: 3 rows, 3 created, 0 skipped, 0 errors
+2026/09/27 21:08:54 POST /uploads/csv 1ms</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>- Every survey order is made hours before the meal: breakfast in the middle of the night, lunch mid-morning, dinner mid-afternoon. Food sits and goes cold or bad.
+- In any kitchen not on UTC, survey scheduling is wrong, and the setting meant to fix it does nothing.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>- Black-box inference: the meal hour seems to be applied to a UTC date and time. The same is likely true for deciding what "today" is: between 8 p.m. and midnight in New York it is already the next day in UTC, so "today" and "tomorrow" would point one day too late. I could not show that here because of the time of day I tested; to be checked.
+- Daylight saving (for example 1 November 2026) should also be tested once this is fixed.</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_csv.py -k kitchen_local_time must pass for breakfast, lunch and dinner (remove the xfail marker once they report XPASS(strict)).
+- Repeat with ORDERHUB_SITE_TZ set to a zone with a different offset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>L37-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>A survey row with an unknown meal is accepted and the order is made immediately</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_csv.py::test_row_with_unknown_meal_is_rejected</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Survey CSV, input validation</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>A row with a meal other than breakfast, lunch or dinner (for example brunch, or a typo like diner) is accepted without an error. It is scheduled for midnight UTC of that day, which is already past, so it is sent to the robot right away.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Survey CSV: "meal is breakfast (made at 8:00), lunch (12:00), or dinner (18:00)".
+- QA_HOMEWORK, Bad data: "OrderHub should be resilient to malformed and adversarial input."</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Upload a survey export with one row whose meal is brunch:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nMia,Brunch,Pancakes,,false,brunch\n'
+2. Wait 3 seconds so the dispatcher can run.
+3. List survey orders:
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -m json.tool
+4. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>- Step 1 returns created 0 and an error for line 2 saying brunch is not a valid meal.
+- No order is created and nothing is sent to the robot.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>- Step 1 returns created 1 and no errors.
+- Step 3: the order's ready_at is today at 00:00:00 UTC and its status is dispatched.
+- Step 4: the robot received the pancakes immediately.</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Upload a survey export with one row whose meal is brunch):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 04:08:57 GMT
+Content-Length: 82
+{"upload_id":"u1790568537472587460","rows":1,"created":1,"skipped":0,"errors":[]}
+Step 3 (List survey orders):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 1,
+            "source": "csv",
+            "external_id": "u1790568537472587460-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Mia",
+            "customer_last": "Brunch",
+            "items": [
+                {
+                    "name": "Pancakes"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "dispatched",
+            "ready_at": "2026-09-28 00:00:00",
+            "created_at": "2026-09-28 04:08:57",
+            "updated_at": "2026-09-28 04:08:57"
+        }
+    ]
+}
+Step 4 (Show what the robot received):
+{"dispatch_id":"698c8fd7f67be54c","order_id":1,"external_ref":"csv:u1790568537472587460-2","source":"csv","station":"assembly-1","customer":"Mia Brunch","items":[{"line":1,"name":"Pancakes","qty":1}],"dispatch_at":"2026-09-28T04:08:57Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/27 21:08:55 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 21:08:55 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 21:08:55 poller: polling http://localhost:8090 every 2s
+2026/09/27 21:08:57 csv upload u1790568537472587460: 1 rows, 1 created, 0 skipped, 0 errors
+2026/09/27 21:08:57 POST /uploads/csv 1ms
+2026/09/27 21:08:57 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>- A typo in the survey (diner, Lunch time, brunch) makes the robot build the order right away instead of at a meal time, with no error to tell anyone the row was wrong.
+- The person who uploaded the file gets "created 1, errors none" and has no reason to check.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>- The upload response already has an errors list, used for rows the CSV reader can't parse. Unknown meal values should be reported there.
+- Related: L37-015 (tomorrow values), L37-004 (webhook fields).</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_csv.py -k unknown_meal must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>L37-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Survey column tomorrow: TRUE, yes or an empty value are silently treated as today</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_csv.py::test_tomorrow_in_capitals_means_tomorrow
+tests/test_csv.py::test_row_with_invalid_tomorrow_value_is_rejected (yes, empty)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Survey CSV, input validation</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Only the exact value true means tomorrow. TRUE, which is how Excel and Google Sheets write booleans, is treated as today, and so are values like yes or an empty cell. No error is reported, so an order meant for tomorrow is made today, and nothing is made tomorrow.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>- README, Payload formats, Survey CSV: "tomorrow (true or false)".
+- README, Pipelines, Survey CSV: "tomorrow says whether the meal is for today or tomorrow."
+- The meal column is already read case-insensitively (Lunch works), so it's inconsistent for tomorrow to be case-sensitive.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Upload a survey export with three dinner rows: tomorrow=TRUE, tomorrow=yes, and tomorrow empty:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nTom,Capitals,Pasta,,TRUE,dinner\nTom,Yes,Pasta,,yes,dinner\nTom,Empty,Pasta,,,dinner\n'
+2. List survey orders and look at ready_at:
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -m json.tool</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>- The TRUE row is scheduled for tomorrow's dinner.
+- The yes and empty rows are rejected with an error for their line, because tomorrow must be true or false.
+- Step 1 returns created 1 and two errors.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>- Step 1 returns created 3 and no errors.
+- Step 2: all three orders are scheduled for today's dinner (today's date at 18:00:00 UTC, see also L37-013). The TRUE row should have been tomorrow.
+- If you run this after today's dinner time has passed, the orders are sent to the robot immediately.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Upload a survey export with three dinner rows):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 04:09:03 GMT
+Content-Length: 82
+{"upload_id":"u1790568543559919007","rows":3,"created":3,"skipped":0,"errors":[]}
+Step 2 (List survey orders and look at ready_at):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 3,
+            "source": "csv",
+            "external_id": "u1790568543559919007-4",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Tom",
+            "customer_last": "Empty",
+            "items": [
+                {
+                    "name": "Pasta"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-28 18:00:00",
+            "created_at": "2026-09-28 04:09:03",
+            "updated_at": "2026-09-28 04:09:03"
+        },
+        {
+            "id": 2,
+            "source": "csv",
+            "external_id": "u1790568543559919007-3",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Tom",
+            "customer_last": "Yes",
+            "items": [
+                {
+                    "name": "Pasta"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-28 18:00:00",
+            "created_at": "2026-09-28 04:09:03",
+            "updated_at": "2026-09-28 04:09:03"
+        },
+        {
+            "id": 1,
+            "source": "csv",
+            "external_id": "u1790568543559919007-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Tom",
+            "customer_last": "Capitals",
+            "items": [
+                {
+                    "name": "Pasta"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-28 18:00:00",
+            "created_at": "2026-09-28 04:09:03",
+            "updated_at": "2026-09-28 04:09:03"
+        }
+    ]
+}
+OrderHub log (GET /api lines not shown):
+2026/09/27 21:09:02 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 21:09:02 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 21:09:02 poller: polling http://localhost:8090 every 2s
+2026/09/27 21:09:03 csv upload u1790568543559919007: 3 rows, 3 created, 0 skipped, 0 errors
+2026/09/27 21:09:03 POST /uploads/csv 1ms</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>- Anyone who edits or exports the survey in Excel or Google Sheets gets TRUE/FALSE, so every "tomorrow" order in that file is made a day early. On the day the customer wanted it, there is nothing.
+- Mistyped values are accepted silently, so the uploader is never told.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>- Related: L37-013 (the time of day is also wrong), L37-014 (unknown meal).</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_csv.py -k tomorrow must pass (remove the xfail markers once they report XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>L37-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>The same survey export uploaded twice at the same time creates duplicate orders</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_csv.py::test_same_export_uploaded_twice_at_once_creates_each_order_once</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Survey CSV, dedup</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Uploading an export twice at once (a double-click on Upload, or a retry after a slow upload timed out) creates many rows twice. With 300 earlier rows already stored, between 25 and 68 of 100 rows became two orders in every run, and each duplicate is made by the robot.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Survey CSV: "Each export contains every response so far, so later uploads repeat earlier rows. Each row becomes one order."
+- README, Order lifecycle: "Each order is dispatched to the robot exactly once."</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. First load 300 survey orders, as if earlier uploads that day already happened. Every upload checks each row against all survey orders already stored, so uploads get slower as more are stored. That makes the problem show up every time:
+{ echo 'first_name,last_name,items,notes,tomorrow,meal'; for i in $(seq 1 300); do echo "Earlier$i,Guest,Soup,,true,dinner"; done; } &gt; /tmp/earlier.csv
+curl -s -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary @/tmp/earlier.csv
+2. Create a new export with 100 rows, all with last name Double:
+{ echo 'first_name,last_name,items,notes,tomorrow,meal'; for i in $(seq 1 100); do echo "Guest$i,Double,Soup,,true,dinner"; done; } &gt; /tmp/export.csv
+3. Upload it twice at the same time:
+curl -s -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary @/tmp/export.csv &amp; curl -s -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary @/tmp/export.csv &amp; wait
+4. Count the orders with last name Double:
+curl -s 'localhost:8080/api/orders?source=csv&amp;limit=1000' | grep -o '"customer_last":"Double"' | wc -l</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>- The two uploads in step 3 together create 100 orders; the second one skips every row.
+- Step 4 prints 100.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>- In step 3, both uploads create orders: their created counts add up to more than 100.
+- Step 4 prints more than 100. Each extra order is a customer's dinner that will be made twice.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (First load 300 survey orders, as if earlier uploads that day already happened):
+{"upload_id":"u1790568546661855918","rows":300,"created":300,"skipped":0,"errors":[]}
+Step 2 (Create a new export with 100 rows, all with last name Double):
+(no output)
+Step 3 (Upload it twice at the same time):
+{"upload_id":"u1790568546871587084","rows":100,"created":57,"skipped":43,"errors":[]}
+{"upload_id":"u1790568546870774036","rows":100,"created":68,"skipped":32,"errors":[]}
+Step 4 (Count the orders with last name Double):
+125
+OrderHub log (GET /api lines not shown):
+2026/09/27 21:09:05 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/27 21:09:05 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/27 21:09:05 poller: polling http://localhost:8090 every 2s
+2026/09/27 21:09:06 csv upload u1790568546661855918: 300 rows, 300 created, 0 skipped, 0 errors
+2026/09/27 21:09:06 POST /uploads/csv 196ms
+2026/09/27 21:09:07 csv upload u1790568546871587084: 100 rows, 57 created, 43 skipped, 0 errors
+2026/09/27 21:09:07 POST /uploads/csv 167ms
+2026/09/27 21:09:07 csv upload u1790568546870774036: 100 rows, 68 created, 32 skipped, 0 errors
+2026/09/27 21:09:07 POST /uploads/csv 175ms
+Automated test (300 earlier rows stored, 100 rows uploaded twice at once): 38 to 68 of 100 rows became two orders, in 8 of 8 runs.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>- A double-click, or an automatic retry after a timeout, duplicates survey orders. Each duplicate is made by the robot.
+- Uploads get slower as the day's exports grow (every row is checked against every stored survey row), so timeouts and retries become more likely exactly when there is more data to duplicate.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>- Black-box inference: each upload checks whether a row was already seen, then creates it. Two uploads running at once both see the row as new.
+- Upload time grows with the number of stored rows: 100 rows took about 0.6 s with none stored and about 1.4 s with 400 stored. To be measured properly in the load tests.
+- Related: L37-010 (duplicate dispatch).</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above several times. Step 4 must print 100 every time.
+- python -m pytest tests/test_csv.py -k twice_at_once must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N13"/>
+  <autoFilter ref="A1:N17"/>
   <conditionalFormatting sqref="D2:D1000">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D2="Critical"</formula>

</xml_diff>

<commit_message>
Bad-data corpus and tests, bugs 017-021
</commit_message>
<xml_diff>
--- a/defects/defects.xlsx
+++ b/defects/defects.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1145,7 +1145,8 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>tests/test_webhook.py::test_webhook_with_missing_fields_is_rejected</t>
+          <t>tests/test_webhook.py::test_webhook_with_missing_fields_is_rejected
+tests/test_bad_data.py::test_webhook_without_an_order_id_is_rejected (comma_in_order_id_key.json, null.json)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1327,8 +1328,9 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Other invalid values are likely accepted too: an unknown order_source, a negative or missing total, an empty items list. These will be covered by the bad-data tests and reported separately if confirmed.
-Related: L37-001 (same outcome: an order merged into another and lost)</t>
+          <t>- The bad-data tests found two more ways to send an order with no order_id, and both are merged into the blank order the same way: a comma in the key ("order_id,": "wh-1" is a key OrderHub doesn't know, so the order has no order_id), and a body that is just null.
+- Other invalid values (an unknown order_source, a negative total, an empty items list) are reported separately as L37-017.
+- Related: L37-001 (same outcome: an order merged into another and lost).</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -3562,8 +3564,784 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>L37-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Webhooks with values outside the spec are accepted: unknown platform, negative total, no items</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_bad_data.py::test_webhook_with_values_outside_the_spec_is_rejected (unknown_platform.json, negative_total.json, no_items.json)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Webhook ingest, input validation</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>OrderHub accepts webhook orders from a platform that isn't Grubstub, DoorDrop or Overeats, orders with a negative total, and orders with an empty items list. All three are sent to the robot. The order with no items reaches the robot as "items": null.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>- README, Payload formats, Webhook: order_source is "The platform: Grubstub, DoorDrop, or Overeats"; total is a number in "Dollars"; items has "One entry per item".
+- QA_HOMEWORK, Bad data: "OrderHub should be resilient to malformed and adversarial input."</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Send an order from a platform OrderHub doesn't work with (UberEats):
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"wh-501","order_source":"UberEats","restaurant":"Just Pizza","first_name":"Uma","last_name":"Park","total":24.5,"items":["Margherita pizza","Garlic knots"],"notes":""}'
+2. Send an order with a negative total:
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"wh-502","order_source":"Grubstub","restaurant":"Just Pizza","first_name":"Nell","last_name":"Park","total":-24.5,"items":["Margherita pizza","Garlic knots"],"notes":""}'
+3. Send an order with an empty items list:
+curl -si -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d '{"order_id":"wh-503","order_source":"Grubstub","restaurant":"Just Pizza","first_name":"Ezra","last_name":"Park","total":24.5,"items":[],"notes":""}'
+4. Wait 3 seconds so the dispatcher can run.
+5. List webhook orders:
+curl -s 'localhost:8080/api/orders?source=webhook' | python3 -m json.tool
+6. Show the counts by platform:
+curl -s localhost:8080/api/stats | python3 -m json.tool
+7. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>- Each request is rejected with 400 and a message naming the invalid field.
+- No orders are created, the stats don't change and nothing is sent to the robot.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>- All three requests return 202.
+- Step 5: three orders, all dispatched: platform UberEats, total -24.5, and an order with no items.
+- Step 6: the stats count an UberEats platform.
+- Step 7: the robot received all three. Ezra's order has "items": null.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Send an order from a platform OrderHub doesn't work with (UberEats)):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 17:31:14 GMT
+Content-Length: 9
+{"id":1}
+Step 2 (Send an order with a negative total):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 17:31:14 GMT
+Content-Length: 9
+{"id":2}
+Step 3 (Send an order with an empty items list):
+HTTP/1.1 202 Accepted
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 17:31:14 GMT
+Content-Length: 9
+{"id":3}
+Step 5 (List webhook orders):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 3,
+            "source": "webhook",
+            "external_id": "wh-503",
+            "platform": "Grubstub",
+            "restaurant": "Just Pizza",
+            "customer_first": "Ezra",
+            "customer_last": "Park",
+            "items": [],
+            "notes": "",
+            "total": 24.5,
+            "status": "dispatched",
+            "ready_at": "2026-09-28 17:31:14",
+            "created_at": "2026-09-28 17:31:14",
+            "updated_at": "2026-09-28 17:31:15"
+        },
+        {
+            "id": 2,
+            "source": "webhook",
+            "external_id": "wh-502",
+            "platform": "Grubstub",
+            "restaurant": "Just Pizza",
+            "customer_first": "Nell",
+            "customer_last": "Park",
+            "items": [
+                {
+                    "name": "Margherita pizza"
+                },
+                {
+                    "name": "Garlic knots"
+                }
+            ],
+            "notes": "",
+            "total": -24.5,
+            "status": "dispatched",
+            "ready_at": "2026-09-28 17:31:14",
+            "created_at": "2026-09-28 17:31:14",
+            "updated_at": "2026-09-28 17:31:15"
+        },
+        {
+            "id": 1,
+            "source": "webhook",
+            "external_id": "wh-501",
+            "platform": "UberEats",
+            "restaurant": "Just Pizza",
+            "customer_first": "Uma",
+            "customer_last": "Park",
+            "items": [
+                {
+                    "name": "Margherita pizza"
+                },
+                {
+                    "name": "Garlic knots"
+                }
+            ],
+            "notes": "",
+            "total": 24.5,
+            "status": "dispatched",
+            "ready_at": "2026-09-28 17:31:14",
+            "created_at": "2026-09-28 17:31:14",
+            "updated_at": "2026-09-28 17:31:15"
+        }
+    ]
+}
+Step 6 (Show the counts by platform):
+{
+    "by_status": {
+        "dispatched": 3
+    },
+    "by_source": {
+        "webhook": 3
+    },
+    "by_platform": {
+        "Grubstub": 2,
+        "UberEats": 1
+    },
+    "total_orders": 3,
+    "total_events": 6,
+    "last_hour": 3,
+    "refreshed_at": "2026-09-28T17:31:15Z"
+}
+Step 7 (Show what the robot received):
+{"dispatch_id":"82688b805a637985","order_id":1,"external_ref":"webhook:wh-501","source":"webhook","station":"assembly-1","customer":"Uma Park","items":[{"line":1,"name":"Margherita pizza","qty":1},{"line":2,"name":"Garlic knots","qty":1}],"dispatch_at":"2026-09-28T17:31:15Z"}
+{"dispatch_id":"02ee4291c64bb092","order_id":2,"external_ref":"webhook:wh-502","source":"webhook","station":"assembly-1","customer":"Nell Park","items":[{"line":1,"name":"Margherita pizza","qty":1},{"line":2,"name":"Garlic knots","qty":1}],"dispatch_at":"2026-09-28T17:31:15Z"}
+{"dispatch_id":"28424db81fcf4fb3","order_id":3,"external_ref":"webhook:wh-503","source":"webhook","station":"assembly-1","customer":"Ezra Park","items":null,"dispatch_at":"2026-09-28T17:31:15Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/28 10:31:13 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/28 10:31:13 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/28 10:31:13 poller: polling http://localhost:8090 every 2s
+2026/09/28 10:31:14 POST /webhooks/orders 1ms
+2026/09/28 10:31:14 POST /webhooks/orders 0s
+2026/09/28 10:31:14 POST /webhooks/orders 0s
+2026/09/28 10:31:15 dispatch: sent 3 orders</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>- The robot is asked to build an order with nothing in it. We don't know how the real cell controller handles "items": null.
+- A misspelled or unknown platform name (Grubhub, doordrop) is made like any other order and counted under a platform that doesn't exist, so per-platform counts are wrong and it isn't clear who to charge or who can cancel it.
+- A negative total goes into the records as if it were real money.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>- The same bad-data tests show what OrderHub does reject correctly with 400: truncated JSON, an empty body, a JSON array instead of an object, total sent as text, and items sent as text (tests/test_bad_data.py::test_webhook_that_cannot_be_read_is_rejected).
+- Accents, emoji, commas, quotes and new lines in names, items and notes reach the robot unchanged (test_special_characters_reach_the_robot_unchanged).
+- Question for the dev team: is a total of 0 valid, for example a free replacement order?
+- Related: L37-004 (missing fields).</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_bad_data.py -k outside_the_spec must pass for all three files (remove the xfail marker once they report XPASS(strict)).
+- Valid orders must still be accepted: python -m pytest -m smoke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="150" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>L37-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>One malformed item in a partner API response loses every order in that response</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_partner_api.py::test_one_malformed_item_does_not_lose_other_orders</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Partner API polling, input validation</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>If one item in a partner response has a value OrderHub can't read (here a price sent as text, "4.25" instead of 4.25), OrderHub throws away the whole response. Every other order in it, including completely valid ones, is never created. Polling then carries on from the next time window, so those orders are never fetched again. The only trace is one line in the OrderHub log.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Partner API: "Nothing that happens upstream may be lost."
+- QA_HOMEWORK, Bad data: "OrderHub should be resilient to malformed and adversarial input."</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Put one response on the partner API with two orders. Order 70000002 (a bagel) is valid. Order 70000003 (a latte) has its price as text:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"item-bagel":{"order":70000002,"name":"Bagel","category":"Food","price":3.5,"status":"ordered"},"item-latte":{"order":70000003,"name":"Latte","category":"Coffee","price":"4.25","status":"ordered"}}}'
+2. Wait 5 seconds so OrderHub polls at least twice.
+3. Put a second, valid order on the partner API, order 70000004 (a muffin):
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"item-muffin":{"order":70000004,"name":"Muffin","category":"Food","price":3,"status":"ordered"}}}'
+4. Wait 5 seconds.
+5. List partner orders:
+curl -s 'localhost:8080/api/orders?source=api' | python3 -m json.tool</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>- Order 70000002 (the bagel) is created and made. One bad item must not stop the rest of the response.
+- The latte item is reported so someone can follow up with the partner. Ideally order 70000003 is created too, or held for review, rather than dropped.
+- Order 70000004 is created.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>- Step 5 shows only order 70000004.
+- Orders 70000002 and 70000003 were never created, although the partner sent them. The bagel order was completely valid.
+- The OrderHub log has one line: "poller: decode: json: cannot unmarshal string into Go struct field APIItem.data.price of type float64". The poll isn't retried and nothing is shown in the UI.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Put one response on the partner API with two orders. Order 70000002 (a bagel) is valid. Order 70000003 (a latte) has its price as text):
+enqueued at 2026-09-28T17:31:20.998497367Z
+Step 3 (Put a second, valid order on the partner API, order 70000004 (a muffin)):
+enqueued at 2026-09-28T17:31:26.009498938Z
+Step 5 (List partner orders):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 1,
+            "source": "api",
+            "external_id": "70000004",
+            "platform": "Partner API",
+            "restaurant": "",
+            "customer_first": "",
+            "customer_last": "",
+            "items": [
+                {
+                    "key": "item-muffin",
+                    "name": "Muffin",
+                    "category": "Food",
+                    "price": 3,
+                    "status": "ordered"
+                }
+            ],
+            "notes": "",
+            "total": 3,
+            "status": "dispatched",
+            "ready_at": "2026-09-28 17:31:27",
+            "created_at": "2026-09-28 17:31:27",
+            "updated_at": "2026-09-28 17:31:28"
+        }
+    ]
+}
+OrderHub log (GET /api lines not shown):
+2026/09/28 10:31:19 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/28 10:31:19 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/28 10:31:19 poller: polling http://localhost:8090 every 2s
+2026/09/28 10:31:21 poller: decode: json: cannot unmarshal string into Go struct field APIItem.data.price of type float64
+2026/09/28 10:31:28 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>- One unexpected value from the partner (a price as text, a null, a new status format) silently drops every order that changed in the same 2-second window. At busy times that is many customers' orders.
+- The partner sees its request succeed, so nobody on either side knows the orders are missing.</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>- Black-box inference: OrderHub reads the whole response in one go and gives up if any value doesn't fit, then moves on to the next time window, as in L37-005.
+- Fixing L37-005 by retrying the failed window is not enough here: the partner would return the same bad item on every retry, polling would be stuck on that window, and no partner orders would arrive at all. The fix has to deal with one bad item without failing the whole response.
+- An item id that contains commas is handled correctly (tests/test_partner_api.py::test_item_id_with_commas_is_kept_as_one_id).
+- The mock partner API only accepts valid JSON, so a truncated or non-JSON response from the partner could not be tested. It most likely behaves like this defect or like L37-005.
+- Related: L37-005.</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_partner_api.py -k malformed_item must pass (remove the xfail marker once it reports XPASS(strict)).
+- Run the step 1 command again without the bad item a few seconds later: new partner orders must keep arriving, so polling is not stuck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="150" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>L37-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>An unterminated quote in a survey CSV silently drops every row after it</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_bad_data.py::test_one_bad_row_does_not_lose_the_other_rows (unterminated_quote.csv)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Survey CSV, parsing</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>When one row has an opening quote without a closing quote, OrderHub reads the rest of the file as part of that row. It reports one error for that row, and every valid row after it is never created and never reported. The response says rows: 1 for a file with 4 rows.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Survey CSV: "Each row becomes one order."
+- QA_HOMEWORK, Bad data: "CSV rows with embedded quotes, commas, and newlines"; "OrderHub should be resilient to malformed and adversarial input."</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Upload a survey export with 4 rows. Bea's row (line 3) opens a quote before Soup and never closes it:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nAl,One,Soup,,true,lunch\nBea,Bad,"Soup,,true,lunch\nCy,Two,Salad,,true,lunch\nDee,Three,Pasta,,true,dinner\n'
+2. List survey orders:
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -m json.tool</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>- Al's, Cy's and Dee's orders are created, and line 3 is listed in errors.
+- Or, if OrderHub can't tell where the broken row ends, the whole upload is rejected with 400, so the file can be fixed and uploaded again (the rows already uploaded would be skipped).
+- Either way, no row disappears without being reported.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>- Step 1 returns 200 with rows 1, created 1 and one error: "line 3: record on line 3; parse error on line 5, column 30: extraneous or missing \" in quoted-field".
+- Step 2 shows only Al's order.
+- Cy's and Dee's rows were not created and are not mentioned anywhere. The response counts 1 row for a file that has 4.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Upload a survey export with 4 rows. Bea's row (line 3) opens a quote before Soup and never closes it):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 17:31:34 GMT
+Content-Length: 184
+{"upload_id":"u1790616694089415063","rows":1,"created":1,"skipped":0,"errors":["line 3: record on line 3; parse error on line 5, column 30: extraneous or missing \" in quoted-field"]}
+Step 2 (List survey orders):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 1,
+            "source": "csv",
+            "external_id": "u1790616694089415063-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Al",
+            "customer_last": "One",
+            "items": [
+                {
+                    "name": "Soup"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 12:00:00",
+            "created_at": "2026-09-28 17:31:34",
+            "updated_at": "2026-09-28 17:31:34"
+        }
+    ]
+}
+OrderHub log (GET /api lines not shown):
+2026/09/28 10:31:32 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/28 10:31:32 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/28 10:31:32 poller: polling http://localhost:8090 every 2s
+2026/09/28 10:31:34 csv upload u1790616694089415063: 1 rows, 1 created, 0 skipped, 1 errors
+2026/09/28 10:31:34 POST /uploads/csv 1ms</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>- Survey customers silently get no meal. The person uploading sees one error for line 3 and has no reason to think the rows after it are gone.
+- Exports are cumulative, so a broken row near the top of the file drops almost the whole day's survey.</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>- Other broken rows are handled well: a quote inside an unquoted field (12" pizza) and a row with too few fields are listed in errors, and the rows around them are created (same test, stray_quote.csv and short_row.csv).
+- Quotes, commas and new lines inside properly quoted fields, Windows line endings and columns in a different order are all read correctly (tests/test_bad_data.py).
+- A simple guard: when the reader stops early, the rows it read plus the errors don't add up to the lines in the file.</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. One of the expected results must hold.
+- python -m pytest tests/test_bad_data.py -k one_bad_row must pass for all three files (remove the xfail marker once unterminated_quote.csv reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="150" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>L37-020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>A survey CSV without the survey columns is accepted: an empty order is sent to the robot and the real orders are lost</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_bad_data.py::test_file_without_the_survey_columns_is_rejected (semicolon_separated.csv, missing_meal_column.csv)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Survey CSV, input validation</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>OrderHub doesn't check that an uploaded file has the survey columns. A file saved with semicolons instead of commas (Excel does this in many European locales) is read as rows with every value empty. The first becomes an empty order that is sent to the robot at once, the rest are skipped as duplicates of it, and every real order in the file is lost. A file without the meal column is also accepted, and its orders are scheduled at midnight UTC instead of a meal time.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>- README, Payload formats, Survey CSV: "Columns: first_name, last_name, items, notes, tomorrow (true or false), meal (breakfast, lunch, or dinner)."
+- README, Pipelines, Survey CSV: "Each row becomes one order."</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Upload a survey export saved with semicolons instead of commas, with Lena's and Marcus's orders:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name;last_name;items;notes;tomorrow;meal\nLena;Cho;Soup;;true;lunch\nMarcus;Reed;Salad;;true;dinner\n'
+2. Upload a survey export that has no meal column, with Nia's order:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow\nNia,Park,Soup,,true\n'
+3. Wait 3 seconds so the dispatcher can run.
+4. List survey orders:
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -m json.tool
+5. Show what the robot received:
+cat data/robot_dispatch.jsonl</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>- Both uploads are rejected with 400 and a message naming the missing columns.
+- No orders are created and nothing is sent to the robot.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>- Step 1 returns 200 with rows 2, created 1, skipped 1 and no errors.
+- Step 4: the order from step 1 has no name and no items, ready_at today at 00:00:00, and status dispatched. Lena's and Marcus's orders don't exist. Marcus's row was counted as skipped, as if it had been uploaded before.
+- Step 2 returns 200 with created 1. Nia's order is scheduled for tomorrow at 00:00:00 UTC (8 p.m. tonight in New York), which is not a meal time.
+- Step 5: the robot received an order with "customer": " " and no items.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Upload a survey export saved with semicolons instead of commas, with Lena's and Marcus's orders):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 17:31:37 GMT
+Content-Length: 82
+{"upload_id":"u1790616697177122518","rows":2,"created":1,"skipped":1,"errors":[]}
+Step 2 (Upload a survey export that has no meal column, with Nia's order):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 17:31:37 GMT
+Content-Length: 82
+{"upload_id":"u1790616697185123015","rows":1,"created":1,"skipped":0,"errors":[]}
+Step 4 (List survey orders):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 2,
+            "source": "csv",
+            "external_id": "u1790616697185123015-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Nia",
+            "customer_last": "Park",
+            "items": [
+                {
+                    "name": "Soup"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 00:00:00",
+            "created_at": "2026-09-28 17:31:37",
+            "updated_at": "2026-09-28 17:31:37"
+        },
+        {
+            "id": 1,
+            "source": "csv",
+            "external_id": "u1790616697177122518-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "",
+            "customer_last": "",
+            "items": [],
+            "notes": "",
+            "total": 0,
+            "status": "dispatched",
+            "ready_at": "2026-09-28 00:00:00",
+            "created_at": "2026-09-28 17:31:37",
+            "updated_at": "2026-09-28 17:31:37"
+        }
+    ]
+}
+Step 5 (Show what the robot received):
+{"dispatch_id":"7aeec86da21eb220","order_id":1,"external_ref":"csv:u1790616697177122518-2","source":"csv","station":"assembly-1","customer":" ","items":null,"dispatch_at":"2026-09-28T17:31:37Z"}
+OrderHub log (GET /api lines not shown):
+2026/09/28 10:31:35 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/28 10:31:35 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/28 10:31:35 poller: polling http://localhost:8090 every 2s
+2026/09/28 10:31:37 csv upload u1790616697177122518: 2 rows, 1 created, 1 skipped, 0 errors
+2026/09/28 10:31:37 POST /uploads/csv 1ms
+2026/09/28 10:31:37 csv upload u1790616697185123015: 1 rows, 1 created, 0 skipped, 0 errors
+2026/09/28 10:31:37 POST /uploads/csv 0s
+2026/09/28 10:31:37 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>- A file in the wrong format turns into an empty order that the robot is asked to build straight away, and every real order in the file is lost.
+- The person uploading gets 200 and "errors": [], so nothing tells them the file was wrong.</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>- Checking the header row is enough to catch this: a file without first_name, last_name, items, tomorrow and meal can't be a survey export.
+- An empty file is already rejected with 400 (same test, empty.csv).
+- Related: L37-014 (unknown meal is made immediately), L37-021 (byte order mark).</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_bad_data.py -k survey_columns must pass for all three files (remove the xfail markers once they report XPASS(strict)).
+- The example export must still upload: python -m pytest -m smoke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="150" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>L37-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>A survey CSV with a byte order mark (Excel "CSV UTF-8") loses first names, and people with the same last name and order are merged</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_bad_data.py::test_file_with_a_byte_order_mark_is_read_correctly</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Survey CSV, parsing, dedup</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Excel's "CSV UTF-8" format starts the file with an invisible byte order mark (BOM). OrderHub then doesn't recognise the first column, first_name, so every order from the file has an empty first name. Because the duplicate check compares names, two people with the same last name who order the same meal (for example two sisters) now look like the same row, and the second one's order is skipped.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Survey CSV: "Each row becomes one order."
+- README, Payload formats, Survey CSV: "Columns: first_name, last_name, ..."</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Upload a survey export that starts with a byte order mark, as Excel's "CSV UTF-8" writes it. Lena and Mia Cho both order soup for lunch; Marcus orders a salad:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'\xef\xbb\xbffirst_name,last_name,items,notes,tomorrow,meal\nLena,Cho,Soup,,true,lunch\nMia,Cho,Soup,,true,lunch\nMarcus,Reed,Salad,,true,dinner\n'
+2. List survey orders:
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -m json.tool
+3. Upload the same three rows without the byte order mark, with the last names changed so they are new rows:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nLena,Choo,Soup,,true,lunch\nMia,Choo,Soup,,true,lunch\nMarcus,Reeds,Salad,,true,dinner\n'</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>- Step 1 returns created 3.
+- Step 2 shows three orders with first names Lena, Mia and Marcus.
+- Step 3 behaves the same as step 1: created 3.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>- Step 1 returns 200 with rows 3, created 2, skipped 1 and no errors.
+- Step 2 shows two orders, both with an empty customer_first. Mia's order was skipped as a duplicate of Lena's.
+- Step 3, the same file without the byte order mark, returns created 3.</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 (Upload a survey export that starts with a byte order mark, as Excel's "CSV UTF-8" writes it. Lena and Mia Cho both order soup for lunch; Marcus orders a salad):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 17:31:43 GMT
+Content-Length: 82
+{"upload_id":"u1790616703279606136","rows":3,"created":2,"skipped":1,"errors":[]}
+Step 2 (List survey orders):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 2,
+            "source": "csv",
+            "external_id": "u1790616703279606136-4",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "",
+            "customer_last": "Reed",
+            "items": [
+                {
+                    "name": "Salad"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 18:00:00",
+            "created_at": "2026-09-28 17:31:43",
+            "updated_at": "2026-09-28 17:31:43"
+        },
+        {
+            "id": 1,
+            "source": "csv",
+            "external_id": "u1790616703279606136-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "",
+            "customer_last": "Cho",
+            "items": [
+                {
+                    "name": "Soup"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-29 12:00:00",
+            "created_at": "2026-09-28 17:31:43",
+            "updated_at": "2026-09-28 17:31:43"
+        }
+    ]
+}
+Step 3 (Upload the same three rows without the byte order mark, with the last names changed so they are new rows):
+HTTP/1.1 200 OK
+Content-Type: application/json
+Date: Mon, 28 Sep 2026 17:31:43 GMT
+Content-Length: 82
+{"upload_id":"u1790616703325291231","rows":3,"created":3,"skipped":0,"errors":[]}
+OrderHub log (GET /api lines not shown):
+2026/09/28 10:31:41 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/28 10:31:41 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/28 10:31:41 poller: polling http://localhost:8090 every 2s
+2026/09/28 10:31:43 csv upload u1790616703279606136: 3 rows, 2 created, 1 skipped, 0 errors
+2026/09/28 10:31:43 POST /uploads/csv 1ms
+2026/09/28 10:31:43 csv upload u1790616703325291231: 3 rows, 3 created, 0 skipped, 0 errors
+2026/09/28 10:31:43 POST /uploads/csv 1ms</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>- Any survey export saved from Excel as "CSV UTF-8" loses every customer's first name, so orders can't be labelled or handed over by name.
+- Family members or colleagues with the same last name who order the same meal lose all but one order, and the upload reports it as an ordinary skipped repeat.</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>- Only the first column is affected. The other columns are found by name as usual.
+- Columns in a different order and header names in capitals are read correctly (tests/test_bad_data.py::test_columns_are_found_by_name_in_any_order).
+- Related: L37-020 (file without the survey columns).</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- python -m pytest tests/test_bad_data.py -k byte_order must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N17"/>
+  <autoFilter ref="A1:N22"/>
   <conditionalFormatting sqref="D2:D1000">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D2="Critical"</formula>

</xml_diff>

<commit_message>
Add inject tool for sending orders by hand. Update to 002, 013, 015
</commit_message>
<xml_diff>
--- a/defects/defects.xlsx
+++ b/defects/defects.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="14520" yWindow="-28300" windowWidth="38880" windowHeight="28300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +11,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$22</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -29,11 +28,14 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -46,7 +48,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -70,36 +72,39 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="00F4B6B6"/>
+          <bgColor rgb="FFDDDDDD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="00F9D3A6"/>
+          <bgColor rgb="FFFBEFA6"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="00FBEFA6"/>
+          <bgColor rgb="FFF9D3A6"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="00DDDDDD"/>
+          <bgColor rgb="FFF4B6B6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -466,11 +471,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="2" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
@@ -479,9 +483,7 @@
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="90" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
-    <col width="55" customWidth="1" min="13" max="13"/>
-    <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="55" customWidth="1" min="12" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -556,7 +558,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="150" customHeight="1">
+    <row r="2" ht="196" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>L37-001</t>
@@ -938,7 +940,7 @@
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>- Black-box inference: same root cause as L37-001. Webhook orders seem to be matched on order_id alone, not platform + order_id.
-- Not yet tested: a cancel from another platform after the order was dispatched. Given L37-001 and the cancel behaviour seen here, it likely flips a dispatched order to cancelled while the robot is building it. To be confirmed in the dispatch tests.
+- Also confirmed after dispatch: a DoorDrop cancel for 2002 sent after Grubstub's order 2002 was dispatched turns that order to cancelled, "by": "DoorDrop", although the robot already built it. Checked by hand with the steps above plus a 3-second wait before step 2; see also L37-011.
 Related: L37-001 (likely same root cause)</t>
         </is>
       </c>
@@ -1472,10 +1474,12 @@
 - Status updates and cancellations in that window are lost too, so a cancelled order may still be made.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>- Black-box inference: after a failed poll, the next poll seems to ask for changes since the time of the failed poll, not since the last successful one. The mock is built to succeed when the same time_since is retried, so a retry would recover everything.
-- Related: restarting OrderHub may lose orders the same way (what happened upstream while it was down). To be tested in the restart tests.</t>
+- Related: restarting OrderHub may lose orders the same way (what happened upstream while it was down). To be tested in the restart tests.
+Every 2 seconds OrderHub asks the partner for everything that changed since the last time it asked. 
+Say the 12:00:02 request gets a 500. The spec says "a retry of the same request succeeds," so OrderHub should ask again with the same time_since=12:00:00. Instead, it has already moved its bookmark forward before the request failed. The next request is "What changed since 12:00:02?", and nobody ever asks about 12:00:00 to 12:00:02 again.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -2947,7 +2951,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Breakfast, lunch and dinner are scheduled at 8:00, 12:00 and 18:00 UTC instead of 8:00, 12:00 and 18:00 in the kitchen's time zone. With the default America/New_York, every survey order is made 4 hours early (5 hours in winter): breakfast at 4 a.m., lunch at 8 a.m., dinner at 2 p.m. Changing -site-tz makes no difference.</t>
+          <t>Breakfast, lunch and dinner are scheduled at 8:00, 12:00 and 18:00 UTC instead of 8:00, 12:00 and 18:00 in the kitchen's time zone. With the default America/New_York, every survey order is made 4 hours early (5 hours in winter): breakfast at 4 a.m., lunch at 8 a.m., dinner at 2 p.m. Changing -site-tz makes no difference. After 8 p.m. in New York (7 p.m. in winter) the day is wrong too: OrderHub is already on the next day in UTC, so today's orders are scheduled for tomorrow and tomorrow's for the day after.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3150,12 +3154,15 @@
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>- Every survey order is made hours before the meal: breakfast in the middle of the night, lunch mid-morning, dinner mid-afternoon. Food sits and goes cold or bad.
-- In any kitchen not on UTC, survey scheduling is wrong, and the setting meant to fix it does nothing.</t>
+- In any kitchen not on UTC, survey scheduling is wrong, and the setting meant to fix it does nothing.
+- Exports uploaded in the evening are scheduled a whole day late: a customer who ordered tomorrow's dinner gets it the day after.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>- Black-box inference: the meal hour seems to be applied to a UTC date and time. The same is likely true for deciding what "today" is: between 8 p.m. and midnight in New York it is already the next day in UTC, so "today" and "tomorrow" would point one day too late. I could not show that here because of the time of day I tested; to be checked.
+          <t>- Black-box inference: the meal hour is applied to a UTC date and time, and "today" is also the UTC date.
+- Confirmed in the evening: on 28 September at 22:38 New York time (02:38 UTC on the 29th), a breakfast row with tomorrow=false was scheduled for 2026-09-29 08:00:00 UTC (4 a.m. the next day in New York), and a dinner row with tomorrow=true for 2026-09-30 18:00:00 UTC, the day after tomorrow.
+- If you run the steps above between 8 p.m. and midnight New York time, the dates in step 2 and step 5 are one day later than written.
 - Daylight saving (for example 1 November 2026) should also be tested once this is fixed.</t>
         </is>
       </c>
@@ -3323,7 +3330,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Only the exact value true means tomorrow. TRUE, which is how Excel and Google Sheets write booleans, is treated as today, and so are values like yes or an empty cell. No error is reported, so an order meant for tomorrow is made today, and nothing is made tomorrow.</t>
+          <t>Only the exact value true means tomorrow. TRUE, which is how Excel and Google Sheets write booleans, is treated as today, and so are values like yes or an empty cell. No error is reported, so an order meant for tomorrow is made a day early, and nothing is made on the day the customer wanted.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3336,43 +3343,44 @@
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
-1. Upload a survey export with three dinner rows: tomorrow=TRUE, tomorrow=yes, and tomorrow empty:
-curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nTom,Capitals,Pasta,,TRUE,dinner\nTom,Yes,Pasta,,yes,dinner\nTom,Empty,Pasta,,,dinner\n'
-2. List survey orders and look at ready_at:
+1. Upload a survey export with four dinner rows: tomorrow=true (to compare with), tomorrow=TRUE, tomorrow=yes, and tomorrow empty:
+curl -si -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nTom,Lower,Pasta,,true,dinner\nTom,Capitals,Pasta,,TRUE,dinner\nTom,Yes,Pasta,,yes,dinner\nTom,Empty,Pasta,,,dinner\n'
+2. List survey orders and compare ready_at:
 curl -s 'localhost:8080/api/orders?source=csv' | python3 -m json.tool</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>- The TRUE row is scheduled for tomorrow's dinner.
+          <t>- The TRUE row (Capitals) has the same ready_at as the true row (Lower): tomorrow's dinner.
 - The yes and empty rows are rejected with an error for their line, because tomorrow must be true or false.
-- Step 1 returns created 1 and two errors.</t>
+- Step 1 returns created 2 and two errors.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>- Step 1 returns created 3 and no errors.
-- Step 2: all three orders are scheduled for today's dinner (today's date at 18:00:00 UTC, see also L37-013). The TRUE row should have been tomorrow.
-- If you run this after today's dinner time has passed, the orders are sent to the robot immediately.</t>
+          <t>- Step 1 returns created 4 and no errors.
+- Step 2: the Capitals, Yes and Empty orders are all scheduled one day earlier than the Lower order. OrderHub treated TRUE, yes and empty as today.
+- The dates themselves are also off because of L37-013, but the one-day difference between true and TRUE is there at any time of day.
+- If today's dinner time has already passed, the TRUE, yes and empty orders are sent to the robot immediately.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Step 1 (Upload a survey export with three dinner rows):
+          <t>Step 1 (Upload a survey export with four dinner rows: tomorrow=true (to compare with), tomorrow=TRUE, tomorrow=yes, and tomorrow empty):
 HTTP/1.1 200 OK
 Content-Type: application/json
-Date: Mon, 28 Sep 2026 04:09:03 GMT
+Date: Tue, 29 Sep 2026 02:39:12 GMT
 Content-Length: 82
-{"upload_id":"u1790568543559919007","rows":3,"created":3,"skipped":0,"errors":[]}
-Step 2 (List survey orders and look at ready_at):
+{"upload_id":"u1790649552052523762","rows":4,"created":4,"skipped":0,"errors":[]}
+Step 2 (List survey orders and compare ready_at):
 {
     "limit": 50,
     "offset": 0,
     "orders": [
         {
-            "id": 3,
+            "id": 4,
             "source": "csv",
-            "external_id": "u1790568543559919007-4",
+            "external_id": "u1790649552052523762-5",
             "platform": "Survey",
             "restaurant": "",
             "customer_first": "Tom",
@@ -3385,14 +3393,14 @@
             "notes": "",
             "total": 0,
             "status": "scheduled",
-            "ready_at": "2026-09-28 18:00:00",
-            "created_at": "2026-09-28 04:09:03",
-            "updated_at": "2026-09-28 04:09:03"
+            "ready_at": "2026-09-29 18:00:00",
+            "created_at": "2026-09-29 02:39:12",
+            "updated_at": "2026-09-29 02:39:12"
         },
         {
-            "id": 2,
+            "id": 3,
             "source": "csv",
-            "external_id": "u1790568543559919007-3",
+            "external_id": "u1790649552052523762-4",
             "platform": "Survey",
             "restaurant": "",
             "customer_first": "Tom",
@@ -3405,14 +3413,14 @@
             "notes": "",
             "total": 0,
             "status": "scheduled",
-            "ready_at": "2026-09-28 18:00:00",
-            "created_at": "2026-09-28 04:09:03",
-            "updated_at": "2026-09-28 04:09:03"
+            "ready_at": "2026-09-29 18:00:00",
+            "created_at": "2026-09-29 02:39:12",
+            "updated_at": "2026-09-29 02:39:12"
         },
         {
-            "id": 1,
+            "id": 2,
             "source": "csv",
-            "external_id": "u1790568543559919007-2",
+            "external_id": "u1790649552052523762-3",
             "platform": "Survey",
             "restaurant": "",
             "customer_first": "Tom",
@@ -3425,18 +3433,38 @@
             "notes": "",
             "total": 0,
             "status": "scheduled",
-            "ready_at": "2026-09-28 18:00:00",
-            "created_at": "2026-09-28 04:09:03",
-            "updated_at": "2026-09-28 04:09:03"
+            "ready_at": "2026-09-29 18:00:00",
+            "created_at": "2026-09-29 02:39:12",
+            "updated_at": "2026-09-29 02:39:12"
+        },
+        {
+            "id": 1,
+            "source": "csv",
+            "external_id": "u1790649552052523762-2",
+            "platform": "Survey",
+            "restaurant": "",
+            "customer_first": "Tom",
+            "customer_last": "Lower",
+            "items": [
+                {
+                    "name": "Pasta"
+                }
+            ],
+            "notes": "",
+            "total": 0,
+            "status": "scheduled",
+            "ready_at": "2026-09-30 18:00:00",
+            "created_at": "2026-09-29 02:39:12",
+            "updated_at": "2026-09-29 02:39:12"
         }
     ]
 }
 OrderHub log (GET /api lines not shown):
-2026/09/27 21:09:02 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
-2026/09/27 21:09:02 orderhub listening on :8080 (site time zone America/New_York)
-2026/09/27 21:09:02 poller: polling http://localhost:8090 every 2s
-2026/09/27 21:09:03 csv upload u1790568543559919007: 3 rows, 3 created, 0 skipped, 0 errors
-2026/09/27 21:09:03 POST /uploads/csv 1ms</t>
+2026/09/28 19:39:10 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/28 19:39:10 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/28 19:39:10 poller: polling http://localhost:8090 every 2s
+2026/09/28 19:39:12 csv upload u1790649552052523762: 4 rows, 4 created, 0 skipped, 0 errors
+2026/09/28 19:39:12 POST /uploads/csv 1ms</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -3447,7 +3475,8 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>- Related: L37-013 (the time of day is also wrong), L37-014 (unknown meal).</t>
+          <t>- The steps compare TRUE with true instead of with a date, because OrderHub's idea of "today" changes in the evening (L37-013). An earlier version of the automated test compared with a date, and passed by accident after 8 p.m. New York time; it now compares with true too.
+- Related: L37-013 (the time of day is also wrong), L37-014 (unknown meal).</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -4343,16 +4372,16 @@
   </sheetData>
   <autoFilter ref="A1:N22"/>
   <conditionalFormatting sqref="D2:D1000">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="3">
       <formula>$D2="Critical"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="2">
       <formula>$D2="High"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="3" dxfId="1">
       <formula>$D2="Medium"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3">
+    <cfRule type="expression" priority="4" dxfId="0">
       <formula>$D2="Low"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Load generator and survey opload growth, two bugs 022 and 023
</commit_message>
<xml_diff>
--- a/defects/defects.xlsx
+++ b/defects/defects.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$24</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,10 @@
     <font>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -64,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -73,6 +77,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -470,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1479,7 +1486,8 @@
           <t>- Black-box inference: after a failed poll, the next poll seems to ask for changes since the time of the failed poll, not since the last successful one. The mock is built to succeed when the same time_since is retried, so a retry would recover everything.
 - Related: restarting OrderHub may lose orders the same way (what happened upstream while it was down). To be tested in the restart tests.
 Every 2 seconds OrderHub asks the partner for everything that changed since the last time it asked. 
-Say the 12:00:02 request gets a 500. The spec says "a retry of the same request succeeds," so OrderHub should ask again with the same time_since=12:00:00. Instead, it has already moved its bookmark forward before the request failed. The next request is "What changed since 12:00:02?", and nobody ever asks about 12:00:00 to 12:00:02 again.</t>
+Say the 12:00:02 request gets a 500. The spec says "a retry of the same request succeeds," so OrderHub should ask again with the same time_since=12:00:00. Instead, it has already moved its bookmark forward before the request failed. The next request is "What changed since 12:00:02?", and nobody ever asks about 12:00:00 to 12:00:02 again.
+- Load test (LOAD_RESULTS.md): with one partner 500 a minute, 1 in 12 partner orders was lost at every load from 100,000 to 1,000,000 orders a day (12 of 144 up to 126 of 1,512). That is the share of partner orders that fall in the poll window of each 500; with orders spread evenly instead of in bursts it would be about 1 in 30.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -2496,7 +2504,9 @@
 - Each attempt gets a new dispatch_id, so the robot cannot de-duplicate on its side.
 - The same happens with a slow robot: with 1.5 seconds per order, 5 orders became 26 builds (one order 8 times). See tests/test_dispatch.py::test_slow_robot_makes_each_order_once.
 - The load test will measure how often this happens at 100,000 requests a day.
-- Related: L37-012 (same timing window lets a cancel be undone).</t>
+- Related: L37-012 (same timing window lets a cancel be undone).
+- Load test (LOAD_RESULTS.md), robot at 30 ms per order: at the expected peak of 100,000 orders a day in bursts of 21 every 5 seconds, no order was made twice. The same 100,000 a day in bursts of 42 every 10 seconds made 54 of 612 webhook orders twice. At 5 times the load, 2,407 of 3,681 orders were made more than once (3,313 extra builds); at 10 times, 7,315 of 7,362 (50,221 extra builds). The threshold is about 34 orders waiting at once: that many take more than a second to send.
+- The same x5 run on a laptop with 16 threads and 32 GB: 2,652 of 3,681 orders made more than once (3,950 extra builds). A bigger machine doesn't help, because the cause is the robot's time per order and the 1-second dispatcher cycle.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -3582,8 +3592,9 @@
       <c r="M17" s="2" t="inlineStr">
         <is>
           <t>- Black-box inference: each upload checks whether a row was already seen, then creates it. Two uploads running at once both see the row as new.
-- Upload time grows with the number of stored rows: 100 rows took about 0.6 s with none stored and about 1.4 s with 400 stored. To be measured properly in the load tests.
-- Related: L37-010 (duplicate dispatch).</t>
+- Upload time grows with the number of stored rows: 100 rows took about 0.6 s with none stored and about 1.4 s with 400 stored.
+- Related: L37-010 (duplicate dispatch).
+- Upload times are measured in L37-023: the bigger the stored survey, the longer the window for a second upload to overlap.</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -4369,8 +4380,222 @@
         </is>
       </c>
     </row>
+    <row r="23" ht="150" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>L37-022</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>A survey upload that takes longer than 15 seconds makes OrderHub use all memory and crash</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>None in the pytest suite: it would crash the OrderHub the other tests share. The big-file case is shown by tools/csv_growth.py (see LOAD_RESULTS.md).</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Survey CSV, availability</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>If a survey upload is still being received after 15 seconds, OrderHub's memory starts growing by more than 100 MB a second and doesn't stop until the system kills it. Two everyday things cause this: a slow connection (a 5-row file sent at 10 bytes a second is enough), or a big cumulative export (on the test machine, about 2,500 rows, because processing an export gets slower with every stored row, see L37-023). While memory grows OrderHub still answers health checks, so nothing looks wrong until it dies. Once it's gone, every pipeline stops: no webhooks accepted, no partner polling, nothing sent to the robot, and it doesn't come back by itself.</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>- README, Capacity: "OrderHub must handle 100,000 requests per day, arriving in bursts rather than evenly."
+- README, Pipelines, Survey CSV: "Survey results are exported and uploaded several times a day. Each export contains every response so far."
+- QA_HOMEWORK, Bad data: "OrderHub should be resilient to malformed and adversarial input."</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+Warning: this makes OrderHub use gigabytes of memory within a minute. On a Mac there is no memory limit, so it keeps growing until you stop it: press Ctrl-C in the make run terminal right after step 4.
+1. Create a small survey export with 5 rows (180 bytes):
+printf 'first_name,last_name,items,notes,tomorrow,meal\nAda,Slow,Soup,,true,dinner\nBo,Slow,Salad,,true,dinner\nCy,Slow,Pasta,,true,dinner\nDi,Slow,Bagel,,true,lunch\nEd,Slow,Juice,,true,lunch\n' &gt; /tmp/slow.csv
+2. Upload it slowly, at 10 bytes a second, like a survey sent over a poor connection. Sending takes about 18 seconds. It runs in the background, and its result line appears later:
+curl -s --limit-rate 10 -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary @/tmp/slow.csv -w '\nupload: HTTP %{http_code} after %{time_total}s\n' &amp;
+3. Show OrderHub's memory every 10 seconds for 90 seconds:
+for i in $(seq 1 9); do sleep 10; P=$(pgrep -x orderhub) &amp;&amp; echo "$(date +%T) OrderHub uses $(( $(ps -o rss= -p $P) / 1024 )) MB" || echo "$(date +%T) OrderHub is not running"; done
+4. Check whether OrderHub still answers:
+curl -sSi -m 5 localhost:8080/healthz</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>- The upload in step 2 succeeds after about 18 seconds with created 5, or is rejected with a clear error if it is too slow.
+- Memory stays at a few tens of MB throughout.
+- Step 4 returns 200. OrderHub keeps working.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>- For the first 15 seconds memory stays at about 10 MB.
+- From then on it grows by about 120 MB a second: 0.7 GB, 1.9 GB, 3.3 GB, 4.7 GB, 5.7 GB, ten seconds apart. OrderHub still answers health checks meanwhile.
+- On the test machine, which limits OrderHub to 6 GB, the system killed it about 70 seconds after the upload started. The upload ended with no response (HTTP 000), step 3 reports "OrderHub is not running", and step 4 can't connect.
+- Only the rows that arrived in the first 15 seconds became orders: Ada's, Bo's and Cy's (checked in the database afterwards). Di's and Ed's were lost, and the person uploading got no response, so there is no way to tell which rows made it.
+- The OrderHub log says nothing about the upload or the error; the last lines are from startup.</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Step 1 (Create a small survey export with 5 rows (180 bytes)):
+(no output)
+Step 2 (Upload it slowly, at 10 bytes a second, like a survey sent over a poor connection. Sending takes about 18 seconds. It runs in the background, and its result line appears later):
+(printed while step 3 was running)
+upload: HTTP 000 after 65.013732s
+Step 3 (Show OrderHub's memory every 10 seconds for 90 seconds):
+10:27:37 OrderHub uses 11 MB
+10:27:47 OrderHub uses 696 MB
+10:27:57 OrderHub uses 1929 MB
+10:28:07 OrderHub uses 3260 MB
+10:28:17 OrderHub uses 4716 MB
+10:28:27 OrderHub uses 5673 MB
+10:28:37 OrderHub is not running
+10:28:47 OrderHub is not running
+10:28:57 OrderHub is not running
+Step 4 (Check whether OrderHub still answers):
+curl: (7) Failed to connect to localhost port 8080 after 0 ms: Couldn't connect to server
+OrderHub log (GET /api and /healthz lines not shown):
+2026/09/29 10:27:25 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/29 10:27:25 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/29 10:27:25 poller: polling http://localhost:8090 every 2s</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>- One slow or large survey upload takes down all of OrderHub. Webhook orders are refused (platforms retry, but only for a while), partner orders stop being fetched, and nothing more is sent to the robot until someone restarts it.
+- Exports are cumulative, so a busy survey reaches the danger size on its own. From then on every upload crashes OrderHub, and re-uploading the file to "try again" crashes it again.
+- There is no warning beforehand: health checks pass until the moment it dies.</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>- Black-box inference: OrderHub gives each request 15 seconds to arrive, and reads the survey file while it is still arriving. After 15 seconds reading fails, and the upload seems to keep retrying the failed read without end, holding on to more memory each time.
+- The big-file case: python -m tools.csv_growth uploads a growing export and stops at the first upload with no answer in 30 seconds. On the 2-core test machine: 2,000 rows took 10.2 s, and the 2,500-row export got no answer. On a laptop with 16 threads and 32 GB: 3,000 rows took 13.8 s, and the 3,500-row export got no answer. A faster machine moves the threshold, but more memory only delays the crash, because memory grows without limit.
+- Found by the load tests, not by reading the source: the first sign was the mock partner API timing out because OrderHub was using all the CPU and memory.
+- Related: L37-023 (upload time grows), L37-016 (duplicates when an upload is retried while the first is still running).</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold, and memory must stay flat for several minutes after the upload.
+- python -m tools.csv_growth must reach 10,000 rows without "no answer after 30 s".
+- The full test suite must still pass: python -m pytest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="150" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>L37-023</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Survey upload time grows with every row ever uploaded: each doubling of the export makes it about 4 times slower</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>tools/csv_growth.py measures it (see LOAD_RESULTS.md). No pass/fail test, because the spec gives no time limit.</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Survey CSV, performance</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Each survey export contains every response so far, and uploading it gets slower much faster than the file grows. On the test machine: 500 rows took 0.7 s, 1,000 rows 2.4 s, 1,500 rows 5.0 s, and 2,000 rows 8.8 s. Four times the rows took about 13 times as long. At around 2,500 rows the upload passes 15 seconds, and then OrderHub crashes (L37-022).</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Survey CSV: "Survey results are exported and uploaded several times a day. Each export contains every response so far, so later uploads repeat earlier rows."
+- README, Capacity: "OrderHub must handle 100,000 requests per day, arriving in bursts rather than evenly."</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder.
+1. Upload the survey export four times as it grows through the day: 500, 1,000, 1,500 and 2,000 rows. Each export has every row so far, and prints how long its upload took:
+for n in 500 1000 1500 2000; do { echo 'first_name,last_name,items,notes,tomorrow,meal'; for i in $(seq 1 $n); do echo "Guest$i,Row,Soup,,true,dinner"; done; } &gt; /tmp/export.csv; curl -s -o /dev/null -w "export of $n rows: HTTP %{http_code} in %{time_total}s\n" -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary @/tmp/export.csv; done</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>- Upload time grows about in line with the file: twice the rows, about twice the time.
+- A few thousand rows upload in well under 15 seconds, so exports keep working as the survey grows.</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>- Each upload is much slower than the one before: 0.7 s, 2.4 s, 5.0 s, 8.8 s on the test machine. Doubling from 1,000 to 2,000 rows made the upload 3.6 times slower.
+- All four uploads return 200, so nothing tells the person uploading that the next export will be the one that fails.</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Step 1 (Upload the survey export four times as it grows through the day: 500, 1,000, 1,500 and 2,000 rows. Each export has every row so far, and prints how long its upload took):
+export of 500 rows: HTTP 200 in 0.667109s
+export of 1000 rows: HTTP 200 in 2.427991s
+export of 1500 rows: HTTP 200 in 4.979792s
+export of 2000 rows: HTTP 200 in 8.843294s
+OrderHub log (GET /api and /healthz lines not shown):
+2026/09/29 10:25:10 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/29 10:25:10 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/29 10:25:10 poller: polling http://localhost:8090 every 2s
+2026/09/29 10:25:12 csv upload u1790702712238516962: 500 rows, 500 created, 0 skipped, 0 errors
+2026/09/29 10:25:12 POST /uploads/csv 666ms
+2026/09/29 10:25:15 csv upload u1790702712919008368: 1000 rows, 500 created, 500 skipped, 0 errors
+2026/09/29 10:25:15 POST /uploads/csv 2.427s
+2026/09/29 10:25:20 csv upload u1790702715365307484: 1500 rows, 500 created, 1000 skipped, 0 errors
+2026/09/29 10:25:20 POST /uploads/csv 4.979s
+2026/09/29 10:25:29 csv upload u1790702720364401383: 2000 rows, 500 created, 1500 skipped, 0 errors
+2026/09/29 10:25:29 POST /uploads/csv 8.843s</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>- A survey that collects a few thousand responses can no longer be uploaded, because exports only grow. At that point uploads crash OrderHub (L37-022).
+- Long uploads widen the window for L37-016: an impatient second click, or a retry after a timeout, lands while the first upload is still running and creates duplicate orders.
+- While an upload runs, OrderHub uses a full CPU core for it. In the load tests the mock partner API stopped answering in time while big uploads were running on the 2-core test machine.</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>- Black-box inference: each row seems to be compared with every survey row stored so far, so the work grows with rows x stored rows.
+- The same growth on a laptop with 16 threads and 32 GB (tools/csv_growth.py): 1,000 rows 1.5 s, 2,000 rows 5.8 s, 3,000 rows 13.8 s, 3,500 rows no answer. Faster, but the same shape: doubling from 1,000 to 2,000 rows made the upload 3.9 times slower.
+- Related: L37-022 (crash past 15 seconds), L37-016 (concurrent uploads duplicate orders).</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>- Run the steps above. The 2,000-row export should take no more than about 4 times as long as the 500-row one.
+- python -m tools.csv_growth must reach 10,000 rows, with upload time growing about in line with the rows.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N22"/>
+  <autoFilter ref="A1:N24"/>
   <conditionalFormatting sqref="D2:D1000">
     <cfRule type="expression" priority="1" dxfId="3">
       <formula>$D2="Critical"</formula>

</xml_diff>

<commit_message>
Add restart tests, 2 more bugs 024 and 025
</commit_message>
<xml_diff>
--- a/defects/defects.xlsx
+++ b/defects/defects.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$26</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1484,7 +1484,7 @@
       <c r="M6" s="3" t="inlineStr">
         <is>
           <t>- Black-box inference: after a failed poll, the next poll seems to ask for changes since the time of the failed poll, not since the last successful one. The mock is built to succeed when the same time_since is retried, so a retry would recover everything.
-- Related: restarting OrderHub may lose orders the same way (what happened upstream while it was down). To be tested in the restart tests.
+- Related: restarting OrderHub loses partner orders the same way, confirmed in L37-024.
 Every 2 seconds OrderHub asks the partner for everything that changed since the last time it asked. 
 Say the 12:00:02 request gets a 500. The spec says "a retry of the same request succeeds," so OrderHub should ask again with the same time_since=12:00:00. Instead, it has already moved its bookmark forward before the request failed. The next request is "What changed since 12:00:02?", and nobody ever asks about 12:00:00 to 12:00:02 again.
 - Load test (LOAD_RESULTS.md): with one partner 500 a minute, 1 in 12 partner orders was lost at every load from 100,000 to 1,000,000 orders a day (12 of 144 up to 126 of 1,512). That is the share of partner orders that fall in the poll window of each 500; with orders spread evenly instead of in bursts it would be about 1 in 30.</t>
@@ -4594,8 +4594,308 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="150" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>L37-024</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Partner orders placed while OrderHub is down are never fetched after it starts again</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_restart.py::test_partner_order_placed_while_orderhub_is_down_arrives_after_restart</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Partner API polling, restart</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>After a restart, OrderHub asks the partner API only for what changed from the moment it started, not since its last successful poll. Everything that happened upstream while it was down is never fetched: new orders, status changes and cancels. OrderHub is down during every deploy, every crash (L37-022) and every reboot, so partner orders are lost each time.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>- README, Pipelines, Partner API: "The response contains every item that changed since time_since ... Nothing that happens upstream may be lost."</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset. Instead of make run, start the mock partner API and OrderHub in two separate terminals, both in the orderhub folder, so OrderHub can be stopped while the mock keeps running (make run always stops both together). These are the same commands make run uses:
+Terminal 1: ./bin/mockapi
+Terminal 2: ./bin/orderhub -db data/orderhub.db -robot-log data/robot_dispatch.jsonl -frontend frontend/dist
+Run the commands below in a third terminal, also in the orderhub folder.
+1. Enqueue partner order 24001 while OrderHub is running:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-24001":{"order":24001,"name":"Cold brew","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"}}}'
+2. Wait 4 seconds, then list partner orders:
+curl -s 'localhost:8080/api/orders?source=api' | python3 -m json.tool
+3. Stop OrderHub: press Ctrl-C in terminal 2. Leave the mock running in terminal 1.
+4. Enqueue partner order 24002, placed upstream while OrderHub is down:
+curl -s -X POST localhost:8090/enqueue -d '{"response":200,"data":{"i-24002":{"order":24002,"name":"Iced tea","category":"Coffee &amp; Tea","price":4.25,"status":"ordered"}}}'
+5. Start OrderHub again in terminal 2, with the same command as before.
+6. Wait 6 seconds, then list partner orders:
+curl -s 'localhost:8080/api/orders?source=api' | python3 -m json.tool
+7. Show what the mock partner API has for today, to confirm order 24002 is there to be fetched:
+curl -s "localhost:8090/orders?time_since=$(date -u +%Y-%m-%dT00:00:00Z)" | python3 -m json.tool</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>- Step 2 lists order 24001.
+- Step 6 lists both 24001 and 24002: after starting again, OrderHub fetches what happened while it was down.</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>- Step 2 lists order 24001, so polling works.
+- Step 6 still lists only 24001. Order 24002 never arrives, however long you wait.
+- Step 7 shows that the mock partner API has order 24002 and would return it for a time_since before the restart. OrderHub simply never asks for that time.</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Step 1 (Enqueue partner order 24001 while OrderHub is running):
+enqueued at 2026-09-30T03:04:19.622325888Z
+Step 2 (Wait 4 seconds, then list partner orders):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 1,
+            "source": "api",
+            "external_id": "24001",
+            "platform": "Partner API",
+            "restaurant": "",
+            "customer_first": "",
+            "customer_last": "",
+            "items": [
+                {
+                    "key": "i-24001",
+                    "name": "Cold brew",
+                    "category": "Coffee &amp; Tea",
+                    "price": 4.25,
+                    "status": "ordered"
+                }
+            ],
+            "notes": "",
+            "total": 4.25,
+            "status": "dispatched",
+            "ready_at": "2026-09-30 03:04:20",
+            "created_at": "2026-09-30 03:04:20",
+            "updated_at": "2026-09-30 03:04:21"
+        }
+    ]
+}
+Step 3 (Stop OrderHub: press Ctrl-C in terminal 2. Leave the mock running in terminal 1):
+(OrderHub stopped with Ctrl-C)
+Step 4 (Enqueue partner order 24002, placed upstream while OrderHub is down):
+enqueued at 2026-09-30T03:04:23.686704903Z
+Step 5 (Start OrderHub again in terminal 2, with the same command as before):
+(OrderHub started again, 3 seconds after step 4)
+Step 6 (Wait 6 seconds, then list partner orders):
+{
+    "limit": 50,
+    "offset": 0,
+    "orders": [
+        {
+            "id": 1,
+            "source": "api",
+            "external_id": "24001",
+            "platform": "Partner API",
+            "restaurant": "",
+            "customer_first": "",
+            "customer_last": "",
+            "items": [
+                {
+                    "key": "i-24001",
+                    "name": "Cold brew",
+                    "category": "Coffee &amp; Tea",
+                    "price": 4.25,
+                    "status": "ordered"
+                }
+            ],
+            "notes": "",
+            "total": 4.25,
+            "status": "dispatched",
+            "ready_at": "2026-09-30 03:04:20",
+            "created_at": "2026-09-30 03:04:20",
+            "updated_at": "2026-09-30 03:04:21"
+        }
+    ]
+}
+Step 7 (Show what the mock partner API has for today, to confirm order 24002 is there to be fetched):
+{
+    "data": {
+        "i-24001": {
+            "order": 24001,
+            "name": "Cold brew",
+            "category": "Coffee &amp; Tea",
+            "price": 4.25,
+            "status": "ordered"
+        },
+        "i-24002": {
+            "order": 24002,
+            "name": "Iced tea",
+            "category": "Coffee &amp; Tea",
+            "price": 4.25,
+            "status": "ordered"
+        }
+    },
+    "response": 200
+}
+OrderHub log, both runs (GET /api lines not shown):
+2026/09/29 20:04:18 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/29 20:04:18 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/29 20:04:18 poller: polling http://localhost:8090 every 2s
+2026/09/29 20:04:21 dispatch: sent 1 orders
+2026/09/29 20:04:26 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/29 20:04:26 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/29 20:04:26 poller: polling http://localhost:8090 every 2s</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>- Every deploy loses the partner orders placed while OrderHub was stopped. A crash loses them for however long it is down, which after L37-022 is until someone notices and restarts it.
+- Status changes and cancels from that time are lost too, so orders can be made after the customer cancelled.
+- The partner sees nothing wrong, and OrderHub logs nothing, so nobody knows which orders are missing.</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>- Black-box inference: the time OrderHub polls from seems to be kept only in memory and set to "now" when it starts. It needs to be stored, and advanced only after a successful poll (the same fix as L37-005).
+- What does survive a restart: orders that were waiting for the robot are sent once each after it starts again (tests/test_restart.py::test_orders_waiting_for_the_robot_are_sent_once_after_restart passes). Webhook orders sent while OrderHub is down fail, and the platforms retry them later.
+- make run can't show this, because stopping it stops the mock too, and a new mock starts empty. That is why the setup starts the two programs separately.
+- Related: L37-005 (a failed poll skips its window, the same kind of loss), L37-022 (a crash that leaves OrderHub down).</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>- Run the steps above. Step 6 must list both orders.
+- python -m pytest tests/test_restart.py must pass (remove the xfail marker once it reports XPASS(strict)).
+- Repeat with OrderHub down for longer (a minute) and with a status change and a cancel enqueued while it is down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="150" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>L37-025</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>An order being sent to the robot when OrderHub crashes is sent again after it starts, so it is built twice</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_restart.py::test_order_being_sent_during_a_crash_is_not_sent_again_after_restart</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Dispatch, restart</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>If OrderHub crashes while the robot is accepting an order, the robot already has the order but OrderHub never records that it was sent. After OrderHub starts again, it sends the same order again, so the robot builds it twice. Each resend has a new dispatch_id, so the robot can't tell it's a repeat from that. Reproduced 3 times out of 3.</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>- README, Order lifecycle: "Each order is dispatched to the robot exactly once."</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Setup: this needs a robot that is slow to accept an order, and OrderHub stopped at a precise moment, which curl can't do. The test harness does both. In the orderhub folder run make build. In the orderhub-qa folder, with the Python environment set up as in its README:
+1. Run the test with its known-bug marker turned off, so it shows the real result. The test makes the robot take 3 seconds to accept orders, sends one webhook order, kills OrderHub (like a crash) as soon as the robot has received it, starts OrderHub again on the same database with a normal robot, and counts how many times the robot received the order:
+python -m pytest tests/test_restart.py -k crash --runxfail -v
+2. Show OrderHub's log of the run: its two starts, and what it recorded as sent:
+grep -E "listening|dispatch" results/orderhub.log</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>- The test passes: the robot receives the order once, before the crash, and it is not sent again after the restart.</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>- The test fails with "the robot received the order 2 times".
+- OrderHub's log shows it starting twice and "dispatch: sent 1 orders" only once, after the restart. The send before the crash left no trace in OrderHub, not even in its log, although the robot had already received the order.</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Step 1 (python -m pytest tests/test_restart.py -k crash --runxfail -v), end of the output:
+services = &lt;harness.services.Services object at 0x7fab998a2fd0&gt;
+    @pytest.mark.xfail(strict=True, reason="L37-025: an order being sent when OrderHub crashes is sent again after restart")
+    def test_order_being_sent_during_a_crash_is_not_sent_again_after_restart(hub, robot, services):
+        robot.delay = 3
+        order_id = hub.post_webhook(webhook_order()).json()["id"]
+        wait_until(lambda: robot.dispatches_for(order_id), message="order never reached the robot")
+        services.stop_orderhub(crash=True)
+        robot.behave()
+        services.start_orderhub()
+        time.sleep(QUIET_SECONDS)
+        count = len(robot.dispatches_for(order_id))
+&gt;       assert count == 1, f"the robot received the order {count} times"
+E       AssertionError: the robot received the order 2 times
+E       assert 2 == 1
+tests/test_restart.py:66: AssertionError
+=========================== short test summary info ============================
+FAILED tests/test_restart.py::test_order_being_sent_during_a_crash_is_not_sent_again_after_restart
+======================= 1 failed, 2 deselected in 5.04s ========================
+Step 2 (grep -E "listening|dispatch" results/orderhub.log):
+2026/09/29 20:04:41 robot: posting dispatches to http://127.0.0.1:18181/dispatch
+2026/09/29 20:04:41 orderhub listening on 127.0.0.1:18080 (site time zone America/New_York)
+2026/09/29 20:04:42 robot: posting dispatches to http://127.0.0.1:18181/dispatch
+2026/09/29 20:04:42 orderhub listening on 127.0.0.1:18080 (site time zone America/New_York)
+2026/09/29 20:04:43 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>- Every hard crash with orders in the middle of being sent makes those orders twice. Crashes are not rare here: L37-022 kills OrderHub whenever a survey upload takes too long.
+- The window is small, about 30 ms per order with a normal robot, but a busy batch keeps it open for longer (a burst of 100 orders takes about 3 seconds to send).</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>- Sending again is the safer of the two possible failures: the alternative is an order that is never made. But the spec says exactly once, so this needs a decision.
+- Question for the team: does the cell controller ignore an order_id it has already built? The order_id is the same in both sends; only dispatch_id changes. If the controller does ignore repeats, keeping dispatch_id the same on a resend (or relying on order_id) fixes this. If not, OrderHub needs to record that an order is being sent before sending it, and check with the controller after a crash.
+- Found by killing OrderHub (kill -9). A normal stop (Ctrl-C) waits for the send to finish and doesn't cause this.
+- Related: L37-010 (orders sent more than once during bursts, a different cause), L37-022 (crash).</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>- Run the steps above. The test must pass, several times in a row.
+- Remove the xfail marker once it reports XPASS(strict).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N24"/>
+  <autoFilter ref="A1:N26"/>
   <conditionalFormatting sqref="D2:D1000">
     <cfRule type="expression" priority="1" dxfId="3">
       <formula>$D2="Critical"</formula>

</xml_diff>

<commit_message>
Add UI tests with Playwright, bufs 026-029
</commit_message>
<xml_diff>
--- a/defects/defects.xlsx
+++ b/defects/defects.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defects'!$A$1:$N$30</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4894,8 +4894,467 @@
         </is>
       </c>
     </row>
+    <row r="27" ht="150" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>L37-026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>The Cancel selected button always shows (0), but still cancels the ticked orders</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_ui.py::test_cancel_button_counts_the_ticked_orders</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>UI, order list</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Ticking orders in the list never changes the button's count: it always reads "Cancel selected (0)". Clicking it still cancels every ticked order. So the one button that cancels orders in bulk tells the operator it will cancel nothing.</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>- README, Order lifecycle: "scheduled or queued orders can be cancelled by an operator".
+- The button's own label promises the number of selected orders.</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. Use a browser for the steps that say so.
+1. Create an order for tomorrow, so it stays scheduled and can be cancelled:
+curl -s -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nAnn,Tick,Soup,,true,dinner\n'
+2. In a browser, open http://localhost:8080.
+3. Tick the checkbox next to Ann Tick's order (#1), and look at the red button above the list.
+4. Click the button.
+5. Check the order's status:
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -c "import json,sys; [print(o['id'], o['customer_first'], o['status']) for o in json.load(sys.stdin)['orders']]"</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>- Step 3: the button reads "Cancel selected (1)".
+- Step 5: Ann's order is cancelled.</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>- Step 3: the button still reads "Cancel selected (0)" after ticking.
+- Step 5: Ann's order is cancelled anyway. The button said 0.</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot after step 3: defects/screenshots/L37-026.png
+Browser steps were done with Playwright in Chromium, time zone America/Los_Angeles. What the page showed is written out below.
+Step 1 (Create an order for tomorrow, so it stays scheduled and can be cancelled):
+{"upload_id":"u1790739233460651407","rows":1,"created":1,"skipped":0,"errors":[]}
+Step 2 (In a browser, open http://localhost:8080):
+(page opened)
+Tabs: All 1, Scheduled 1, Queued 0, Dispatched 0, Cancelled 0
+Rows:
+| #1 |  Ann Tick Survey | Survey upload | 1 | — | Oct 1, 6:00 PM | Scheduled
+Step 3 (Tick the checkbox next to Ann Tick's order (#1), and look at the red button above the list):
+Ticks: #1 ticked
+Button: Cancel selected (0)
+Step 4 (Click the button):
+(clicked)
+Step 5 (Check the order's status):
+1 Ann cancelled
+OrderHub log (GET /api lines not shown):
+2026/09/29 20:33:51 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/29 20:33:51 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/29 20:33:51 poller: polling http://localhost:8090 every 2s
+2026/09/29 20:33:53 csv upload u1790739233460651407: 1 rows, 1 created, 0 skipped, 0 errors
+2026/09/29 20:33:53 POST /uploads/csv 1ms
+2026/09/29 20:33:53 GET / 12ms
+2026/09/29 20:33:53 GET /assets/index-D0NAr4zk.js 0s
+2026/09/29 20:33:53 GET /assets/index-AFcjEMGe.css 0s
+2026/09/29 20:33:55 POST /api/orders/1/cancel 0s</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>- An operator can't see how many orders a click will cancel. With several ticked, "(0)" suggests nothing will happen, and then they are all cancelled.
+- An operator who thinks the ticking didn't work may click again, or tick more.</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>- Found by hand first (my own notes while exploring the UI), then automated.
+- Black-box inference: the ticked orders are remembered (the click cancels them), only the count on the button isn't updated.
+- Related: L37-027 (the tick can move to a different order).</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold, with 1, 2 and 0 orders ticked.
+- python -m pytest tests/test_ui.py -k counts must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="150" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>L37-027</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>When a new order arrives, the tick moves to a different order, and Cancel selected cancels one that isn't ticked on screen</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_ui.py::test_tick_stays_on_the_same_order_when_a_new_order_arrives</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>UI, order list, cancel</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>The order list refreshes every 3 seconds with the newest order at the top. When a new order arrives, each tick stays at the same row position instead of staying with its order, so it now shows next to a different order. Cancel selected still cancels the order that was originally ticked. The operator sees one order ticked and cancels another.</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>- README, Order lifecycle: "scheduled or queued orders can be cancelled by an operator".
+- README, Pipelines, Webhook: "Traffic is bursty." New orders arrive while operators are working in the list.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. Use a browser for the steps that say so.
+1. Create two orders for tomorrow, Ann (#1) and Cy (#2):
+curl -s -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nAnn,Tick,Soup,,true,dinner\nCy,Tick,Soup,,true,dinner\n'
+2. In a browser, open http://localhost:8080. Cy is at the top, Ann below.
+3. Tick Ann's order (#1).
+4. With the page still open, create one more order, Ben (#3):
+curl -s -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nBen,Tick,Soup,,true,dinner\n'
+5. Wait until Ben's order appears at the top of the list (up to 3 seconds), and look at which order is ticked.
+6. Click Cancel selected.
+7. Check which order was cancelled:
+curl -s 'localhost:8080/api/orders?source=csv' | python3 -c "import json,sys; [print(o['id'], o['customer_first'], o['status']) for o in json.load(sys.stdin)['orders']]"</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>- Step 5: Ann's order is still ticked, wherever it is in the list.
+- Step 7: Ann's order is cancelled, and nothing else.</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>- Step 5: the tick is now next to Cy's order (#2), in the row where Ann's order was. Ann's order (#1), now one row lower, is not ticked.
+- Step 7: Ann's order is cancelled, although the screen showed Cy ticked. Cy's order, the one shown ticked, is not cancelled.</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot at step 5: defects/screenshots/L37-027.png
+Browser steps were done with Playwright in Chromium, time zone America/Los_Angeles. What the page showed is written out below.
+Step 1 (Create two orders for tomorrow, Ann (#1) and Cy (#2)):
+{"upload_id":"u1790739242583567503","rows":2,"created":2,"skipped":0,"errors":[]}
+Step 2 (In a browser, open http://localhost:8080. Cy is at the top, Ann below):
+(page opened)
+Tabs: All 2, Scheduled 2, Queued 0, Dispatched 0, Cancelled 0
+Rows:
+| #2 |  Cy Tick Survey | Survey upload | 1 | — | Oct 1, 6:00 PM | Scheduled
+| #1 |  Ann Tick Survey | Survey upload | 1 | — | Oct 1, 6:00 PM | Scheduled
+Step 3 (Tick Ann's order (#1)):
+Ticks: #2 not ticked, #1 ticked
+Button: Cancel selected (0)
+Step 4 (With the page still open, create one more order, Ben (#3)):
+{"upload_id":"u1790739244458346190","rows":1,"created":1,"skipped":0,"errors":[]}
+Step 5 (Wait until Ben's order appears at the top of the list (up to 3 seconds), and look at which order is ticked):
+Rows:
+| #3 |  Ben Tick Survey | Survey upload | 1 | — | Oct 1, 6:00 PM | Scheduled
+| #2 |  Cy Tick Survey | Survey upload | 1 | — | Oct 1, 6:00 PM | Scheduled
+| #1 |  Ann Tick Survey | Survey upload | 1 | — | Oct 1, 6:00 PM | Scheduled
+Ticks: #3 not ticked, #2 ticked, #1 not ticked
+Button: Cancel selected (0)
+Step 6 (Click Cancel selected):
+(clicked)
+Step 7 (Check which order was cancelled):
+3 Ben scheduled
+2 Cy scheduled
+1 Ann cancelled
+OrderHub log (GET /api lines not shown):
+2026/09/29 20:34:01 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/29 20:34:01 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/29 20:34:01 poller: polling http://localhost:8090 every 2s
+2026/09/29 20:34:02 csv upload u1790739242583567503: 2 rows, 2 created, 0 skipped, 0 errors
+2026/09/29 20:34:02 POST /uploads/csv 1ms
+2026/09/29 20:34:02 GET / 2ms
+2026/09/29 20:34:02 GET /assets/index-D0NAr4zk.js 1ms
+2026/09/29 20:34:02 GET /assets/index-AFcjEMGe.css 0s
+2026/09/29 20:34:04 csv upload u1790739244458346190: 1 rows, 1 created, 0 skipped, 0 errors
+2026/09/29 20:34:04 POST /uploads/csv 0s
+2026/09/29 20:34:06 POST /api/orders/1/cancel 1ms</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>- An operator cancels the wrong customer's order: the customer they meant to cancel gets their food, and a customer who never cancelled gets nothing.
+- During a busy period new orders arrive every few seconds, so this happens whenever an operator takes more than a moment between ticking and clicking.
+- Nothing on screen shows it happened. Together with L37-026, the operator can't check what the click will do.</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>- Black-box inference: rows seem to be matched by their position in the list rather than by order id when the list refreshes.
+- Related: L37-026 (Cancel selected shows 0).</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold.
+- Also tick an order, let two or three new orders arrive, untick and tick again, then cancel: only the order ticked on screen may be cancelled.
+- python -m pytest tests/test_ui.py -k tick must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="150" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>L37-028</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>The status tab counts never change after the page loads</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_ui.py::test_status_tab_counts_update_when_orders_arrive</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>UI, status tabs</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>The counts next to All, Scheduled, Queued, Dispatched and Cancelled show the numbers from when the page was opened. The order list below keeps refreshing every 3 seconds, but the counts don't change until the page is reloaded.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>- README, OrderHub API: GET /api/stats returns "Counts by status, source, and platform", which is what the tabs show.</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. Use a browser for the steps that say so.
+1. Create two orders for tomorrow:
+curl -s -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nAnn,Tick,Soup,,true,dinner\nCy,Tick,Soup,,true,dinner\n'
+2. In a browser, open http://localhost:8080 and look at the counts in the status tabs on the left.
+3. With the page still open, create three more orders:
+curl -s -X POST localhost:8080/uploads/csv -H 'Content-Type: text/csv' --data-binary $'first_name,last_name,items,notes,tomorrow,meal\nDee,Tick,Soup,,true,dinner\nEve,Tick,Soup,,true,dinner\nFay,Tick,Soup,,true,dinner\n'
+4. Wait 10 seconds. The list now shows 5 orders. Look at the tab counts again.
+5. Reload the page and look at the tab counts.</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>- Step 4: the tabs show All 5 and Scheduled 5, matching the list.</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>- Step 2: All 2, Scheduled 2, which is correct.
+- Step 4: still All 2 and Scheduled 2, although the list shows 5 orders and the API's stats say 5.
+- Step 5: after reloading, All 5 and Scheduled 5.</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot at step 4: defects/screenshots/L37-028.png
+Browser steps were done with Playwright in Chromium, time zone America/Los_Angeles. What the page showed is written out below.
+Step 1 (Create two orders for tomorrow):
+{"upload_id":"u1790739254005894287","rows":2,"created":2,"skipped":0,"errors":[]}
+Step 2 (In a browser, open http://localhost:8080 and look at the counts in the status tabs on the left):
+(page opened)
+Tabs: All 2, Scheduled 2, Queued 0, Dispatched 0, Cancelled 0
+Rows:
+| #2 |  Cy Tick Survey | Survey upload | 1 | — | Oct 1, 6:00 PM | Scheduled
+| #1 |  Ann Tick Survey | Survey upload | 1 | — | Oct 1, 6:00 PM | Scheduled
+Step 3 (With the page still open, create three more orders):
+{"upload_id":"u1790739255143756453","rows":3,"created":3,"skipped":0,"errors":[]}
+Step 4 (Wait 10 seconds. The list now shows 5 orders. Look at the tab counts again):
+Tabs: All 2, Scheduled 2, Queued 0, Dispatched 0, Cancelled 0
+Rows shown: 5
+Top bar: Updated Sep 29, 8:34 PM
+API stats: {"by_status":{"scheduled":5},"by_source":{"csv":5},"by_platform":{"Survey":5},"total_orders":5,"total_events":10,"last_hour":5,"refreshed_at":"2026-09-30T03:34:15Z"}
+Step 5 (Reload the page and look at the tab counts):
+Tabs: All 5, Scheduled 5, Queued 0, Dispatched 0, Cancelled 0
+OrderHub log (GET /api lines not shown):
+2026/09/29 20:34:12 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/29 20:34:12 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/29 20:34:12 poller: polling http://localhost:8090 every 2s
+2026/09/29 20:34:14 csv upload u1790739254005894287: 2 rows, 2 created, 0 skipped, 0 errors
+2026/09/29 20:34:14 POST /uploads/csv 1ms
+2026/09/29 20:34:14 GET / 2ms
+2026/09/29 20:34:14 GET /assets/index-AFcjEMGe.css 0s
+2026/09/29 20:34:14 GET /assets/index-D0NAr4zk.js 3ms
+2026/09/29 20:34:15 csv upload u1790739255143756453: 3 rows, 3 created, 0 skipped, 0 errors
+2026/09/29 20:34:15 POST /uploads/csv 1ms
+2026/09/29 20:34:25 GET / 0s
+2026/09/29 20:34:25 GET /assets/index-D0NAr4zk.js 0s
+2026/09/29 20:34:25 GET /assets/index-AFcjEMGe.css 0s</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>- An operator watching the Queued count during a rush sees a number from whenever they opened the page. Orders can pile up (for example while the robot is slow, see L37-010) while the tab shows 0.
+- The page looks live (the list refreshes, and the top bar says "Updated" with the current time), so there is no reason to suspect the counts.</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>- The refresh itself works: the API's /api/stats returns the new counts at every refresh. Only the tabs don't show them.</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>- Run the steps above. All expected results must hold without reloading.
+- python -m pytest tests/test_ui.py -k tab_counts must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="150" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>L37-029</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Make at shows the UTC time as if it were local time</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_ui.py::test_make_at_is_shown_in_local_time</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>UI, order list and order page</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>OrderHub's API gives ready_at in UTC without saying so ("2026-09-30 03:34:29"). The UI shows that time as if it were the operator's local time. In California (UTC-7) an order made at 8:34 PM shows as "Sep 30, 3:34 AM", the next morning. It also hides L37-013: a survey dinner scheduled at 18:00 UTC shows as 6:00 PM, which looks right, although the kitchen makes it at 2:00 PM New York time.</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>- README, Order lifecycle: "Every order has a ready_at: the earliest time it may be sent to the robot."
+- README, Pipelines, Survey CSV: meal times are "in the kitchen's local time zone".</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Setup: in the orderhub folder, run make reset, then make run. Leave it running and run the commands below in a second terminal, also in the orderhub folder. Use a browser for the steps that say so.
+1. Send a webhook order. It is made right away:
+curl -s -X POST localhost:8080/webhooks/orders -H 'Content-Type: application/json' -d @data/examples/webhook/new_order.json
+2. Show the order's ready_at, the time it may be made, as the API gives it (UTC):
+curl -s localhost:8080/api/orders/1 | python3 -m json.tool | grep ready_at
+3. In a browser, open http://localhost:8080 and look at the order's Make at column. Compare it with the time on your computer.</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>- Step 3: Make at shows the time the order was sent in, in the browser's time zone, for example the current time.</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>- Step 2: ready_at is in UTC, with no time zone marked.
+- Step 3: Make at shows exactly the UTC clock time, labelled as local time: 7 hours ahead in California (and the next day in the evening), 4 hours ahead in New York in summer.</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Screenshot at step 3: defects/screenshots/L37-029.png
+Browser steps were done with Playwright in Chromium, time zone America/Los_Angeles. What the page showed is written out below.
+Step 1 (Send a webhook order. It is made right away):
+{"id":1}
+Step 2 (Show the order's ready_at, the time it may be made, as the API gives it (UTC)):
+"ready_at": "2026-09-30 03:34:29",
+Step 3 (In a browser, open http://localhost:8080 and look at the order's Make at column. Compare it with the time on your computer):
+(page opened)
+Tabs: All 1, Scheduled 0, Queued 1, Dispatched 0, Cancelled 0
+Rows:
+| #1 |  Ada Park Just Pizza | Delivery app | 2 | $24.5 | Sep 30, 3:34 AM | Queued
+Browser time now: 9/29/2026, 8:34:30 PM (America/Los_Angeles)
+Order page: Customer Ada Park Restaurant Just Pizza Make at Sep 30, 3:34 AM Total $24.5 | History: Received Sep 30, 3:34 AM Sent to robot Sep 30, 3:34 AM
+OrderHub log (GET /api lines not shown):
+2026/09/29 20:34:27 robot: simulated, writing dispatches to data/robot_dispatch.jsonl
+2026/09/29 20:34:27 orderhub listening on :8080 (site time zone America/New_York)
+2026/09/29 20:34:27 poller: polling http://localhost:8090 every 2s
+2026/09/29 20:34:29 POST /webhooks/orders 1ms
+2026/09/29 20:34:29 GET / 3ms
+2026/09/29 20:34:29 GET /assets/index-D0NAr4zk.js 0s
+2026/09/29 20:34:29 GET /assets/index-AFcjEMGe.css 0s
+2026/09/29 20:34:29 dispatch: sent 1 orders</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>- Operators see wrong times for every order: live orders look as if they are hours in the future, and survey orders look as if they are made at the right meal time when they are not.
+- It hides L37-013 from the people most likely to notice it: the kitchen staff looking at the screen.</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>- The same happens on the order page (Make at) and in the history times.
+- The fix can be on either side: the API could return times with a time zone (for example 2026-09-30T03:36:40Z), or the UI could treat them as UTC.
+- Related: L37-013 (survey meals scheduled in UTC).</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>- Run the steps above in two browser time zones. Make at must match the local time in each.
+- python -m pytest tests/test_ui.py -k local_time must pass (remove the xfail marker once it reports XPASS(strict)).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N26"/>
+  <autoFilter ref="A1:N30"/>
   <conditionalFormatting sqref="D2:D1000">
     <cfRule type="expression" priority="1" dxfId="3">
       <formula>$D2="Critical"</formula>

</xml_diff>